<commit_message>
fix: address CodeRabbit review comments
</commit_message>
<xml_diff>
--- a/tools/excel/soc-cmm/soc-cmm-2.4.2-basic.xlsx
+++ b/tools/excel/soc-cmm/soc-cmm-2.4.2-basic.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Nadia QOUDHADH</t>
+          <t>Nadia Qoudhadh</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,11 @@
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -848,7 +852,13 @@
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Avez-vous identifié les principaux moteurs métier?</t>
+          <t>Avez-vous identifié les principaux moteurs métier?
+Maturity guidance:
+1 - Business drivers are unknown
+2 - Basic awareness of business drivers
+3 - Some business drivers have been identified
+4 - Most business drivers have been identified
+5 - All business drivers are well known within the SOC</t>
         </is>
       </c>
     </row>
@@ -881,7 +891,13 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Avez-vous documenté les principaux moteurs métier?</t>
+          <t>Avez-vous documenté les principaux moteurs métier?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of business drivers
+4 - Single document, full description of business drivers
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -914,7 +930,13 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Utilisez-vous les moteurs métier dans le processus de prise de décision?</t>
+          <t>Utilisez-vous les moteurs métier dans le processus de prise de décision?
+Maturity guidance:
+1 - Business drivers are not part of decision making
+2 - Business drivers are referred to on an ad-hoc basis
+3 - Business drivers are occasionally used in decisions
+4 - Business drivers are used in most decisions
+5 - Business drivers are used in all relevant decisions</t>
         </is>
       </c>
     </row>
@@ -947,7 +969,13 @@
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Vérifiez-vous régulièrement si le catalogue de services actuel is aligné avec les moteurs métier?</t>
+          <t>Vérifiez-vous régulièrement si le catalogue de services actuel is aligné avec les moteurs métier?
+Maturity guidance:
+1 - Service catalogue has not been checked for alignment
+2 - Alignment is performed on an ad-hoc basis
+3 - Alignment was performed but not maintained
+4 - Alignment is performed and maintained regularly
+5 - Every change in the catalogue is checked against drivers</t>
         </is>
       </c>
     </row>
@@ -980,7 +1008,13 @@
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Les moteurs métier ont-ils ont été validés avec les parties prenantes métier?</t>
+          <t>Les moteurs métier ont-ils ont été validés avec les parties prenantes métier?
+Maturity guidance:
+1 - Business drivers have not been validated
+2 - Basic awareness of SOC drivers exists among stakeholders
+3 - Stakeholders informally informed of business drivers
+4 - Alignment of SOC drivers with stakeholders is performed
+5 - Business drivers are formally validated by stakeholders</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1070,13 @@
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Avez-vous identifié les clients &amp; parties prenantes du SOC?</t>
+          <t>Avez-vous identifié les clients &amp; parties prenantes du SOC?
+Maturity guidance:
+1 - SOC customers are not known
+2 - Basic awareness of SOC customers
+3 - Some customers have been identified
+4 - Customers have mostly been identified
+5 - All customers are identified, including relevance and context</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1348,13 @@
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Avez-vous documenté the main SOC les clients &amp; parties prenantes?</t>
+          <t>Avez-vous documenté the main SOC les clients &amp; parties prenantes?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of SOC customers
+4 - Single document, full description of SOC customers
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1387,13 @@
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Différenciez-vous output towards these specific les clients &amp; parties prenantes?</t>
+          <t>Différenciez-vous output towards these specific les clients &amp; parties prenantes?
+Maturity guidance:
+1 - Output is the same for all customers
+2 - Output is somewhat contextualized
+3 - Some customers receive differentiated output
+4 - All important customers receive differentiated output
+5 - All customers receive specific output based on context and type</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1426,13 @@
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Avez-vous des accords de niveau de service agreements with these les clients &amp; parties prenantes?</t>
+          <t>Avez-vous des accords de niveau de service agreements with these les clients &amp; parties prenantes?
+Maturity guidance:
+1 - Contractual agreements not in place
+2 - No contract in place, ad-hoc agreements made
+3 - Basic contract in place, not formally signed of
+4 - Contract signed, but not regularly reviewed
+5 - Contract signed, approved by- and regularly reviewed with customers</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1465,13 @@
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Envoyez-vous régulièrement updates to your les clients &amp; parties prenantes?</t>
+          <t>Envoyez-vous régulièrement updates to your les clients &amp; parties prenantes?
+Maturity guidance:
+1 - No updates sent to customers
+2 - Ad-hoc updates sent to some customers
+3 - Frequent updates sent to most customers
+4 - Periodical updates sent to all customers
+5 - Periodical updates sent and discussed with all customers</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1504,13 @@
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Mesurez-vous et gérez-vous activement and manage customer &amp; stakeholder satisfaction?</t>
+          <t>Mesurez-vous et gérez-vous activement and manage customer &amp; stakeholder satisfaction?
+Maturity guidance:
+1 - Customer satisfaction not measured or managed
+2 - Customer satisfaction managed in ad-hoc fashion
+3 - Customer satisfaction metrics defined, not applied structurally
+4 - Customer satisfaction measured structurally, not actively managed
+5 - Customer satisfaction fully managed and improved over time</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1566,13 @@
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Le SOC have a formal charter document en place?</t>
+          <t>Le SOC have a formal charter document en place?
+Maturity guidance:
+1 - No charter document in place
+2 - Some ad-hoc information across documents
+3 - Basic charter document created
+4 - Single charter, full description of SOC strategic elements
+5 - Charter completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1925,13 @@
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Le SOC est-il charter document regularly updated?</t>
+          <t>Le SOC est-il charter document regularly updated?
+Maturity guidance:
+1 - Charter is never updated
+2 - Charter is updated on ad-hoc basis
+3 - Charter is updated on major changes in business strategy
+4 - Charter is regularly updated
+5 - Charter periodically updated and realigned with business strategy</t>
         </is>
       </c>
     </row>
@@ -1882,7 +1964,13 @@
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Le SOC est-il charter document approved by the business / CISO?</t>
+          <t>Le SOC est-il charter document approved by the business / CISO?
+Maturity guidance:
+1 - Charter is not approved
+2 - Business / CISO has basic awareness of the charter
+3 - Business / CISO has full awareness of the charter
+4 - Business / CISO approves of the content, but not formally
+5 - Charter is formally approved by the business / CISO</t>
         </is>
       </c>
     </row>
@@ -1915,7 +2003,13 @@
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Tous les parties prenantes familiar avec le SOC charter document contents?</t>
+          <t>Tous les parties prenantes familiar avec le SOC charter document contents?
+Maturity guidance:
+1 - Stakeholders are unfamiliar with the charter
+2 - Some stakeholders are aware of the charter, but not its contents
+3 - Some stakeholders are aware of the charter and its contents
+4 - All stakeholders are aware, not all stakeholders know its contents
+5 - All Stakeholders are aware of the charter and its contents</t>
         </is>
       </c>
     </row>
@@ -1971,7 +2065,13 @@
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Le SOC have a governance process en place?</t>
+          <t>Le SOC have a governance process en place?
+Maturity guidance:
+1 - SOC governance process is not in place
+2 - SOC governance is done in an ad-hoc fashion
+3 - Several governance elements are in place, but not structurally
+4 - Formal governance process is in place that covers most SOC aspects
+5 - Formal governance process is in place and covers all SOC aspects</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2104,13 @@
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Have all governance elements been identified?</t>
+          <t>Have all governance elements been identified?
+Maturity guidance:
+1 - No governance elements have been identified
+2 - Some governance elements are identified and governed ad-hoc
+3 - Some governance elements are identified and governed actively
+4 - Most governance elements are identified and actively governed
+5 - All elements are identified and actively governed</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2544,13 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Is cost management en place?</t>
+          <t>Is cost management en place?
+Maturity guidance:
+1 - Cost management not in place
+2 - Costs visible, basic budget allocation in place
+3 - Costs fully visible and mostly managed, forecasting in place
+4 - Costs fully managed, not formally aligned with business stakeholders
+5 - Costs fully managed and formally aligned with business stakeholders</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2822,13 @@
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Tous les governance elements formellement documenté?</t>
+          <t>Tous les governance elements formellement documenté?
+Maturity guidance:
+1 - No governance document in place
+2 - Some ad-hoc information across documents
+3 - Basic governance document created
+4 - Single document, full description of governance elements
+5 - Governance document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2861,13 @@
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Are SOC governance meetings regularly held?</t>
+          <t>Are SOC governance meetings regularly held?
+Maturity guidance:
+1 - No governance meetings held
+2 - Governance meetings held in an ad-hoc fashion
+3 - Governance meetings regularly scheduled
+4 - Governance meetings at different levels scheduled and structured
+5 - Governance meetings at different levels scheduled, ToR formalised</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2900,13 @@
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Is the governance process régulièrement revu?</t>
+          <t>Is the governance process régulièrement revu?
+Maturity guidance:
+1 - Governance process is not reviewed
+2 - Governance process is reviewed in an ad-hoc fashion
+3 - Process is reviewed using a structured approach in an ad-hoc fashion
+4 - Process is regularly and informally reviewed and updated
+5 - Process is regularly and formally reviewed and updated with findings</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2939,13 @@
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Is the governance process aligné avec toutes les parties prenantes?</t>
+          <t>Is the governance process aligné avec toutes les parties prenantes?
+Maturity guidance:
+1 - Stakeholders are unfamiliar with the process
+2 - Some stakeholders are aware of the process, but not its details
+3 - Some stakeholders are aware of the process and its details
+4 - All stakeholders are aware, not all stakeholders know its details
+5 - All stakeholders are aware of the process and its details</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2978,13 @@
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Le SOC est-il regularly audited or subjected to (external) assessments?</t>
+          <t>Le SOC est-il regularly audited or subjected to (external) assessments?
+Maturity guidance:
+1 - No assessments are performed
+2 - The SOC is assessed in an ad-hoc fashion
+3 - The SOC is assessed using a structured approach in an ad-hoc fashion
+4 - The SOC is regularly and informally assessed
+5 - The SOC is regularly and formally assessed by a third party</t>
         </is>
       </c>
     </row>
@@ -2875,7 +3017,13 @@
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)n active cooperation with other SOCs (external)?</t>
+          <t>Y a-t-il un(e)n active cooperation with other SOCs (external)?
+Maturity guidance:
+1 - No cooperation with other SOCs
+2 - Some ad-hoc informal information exchange
+3 - Regular exchange with external SOCs, no defined process
+4 - Defined process for information exchange, regular exchange in place
+5 - Continuous formalized active cooperation and information exchange</t>
         </is>
       </c>
     </row>
@@ -2931,7 +3079,13 @@
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)n information security policy en place that supports le SOC activities?</t>
+          <t>Y a-t-il un(e)n information security policy en place that supports le SOC activities?
+Maturity guidance:
+1 - No formal information security policy in place
+2 - Information security policy in place, no mention of SOC activities
+3 - Policy in place, SOC activities mentioned without mandate
+4 - Policy in place, SOC activities mentioned in detail with mandate
+5 - Policy with SOC activities and mandate in place, actively communicated</t>
         </is>
       </c>
     </row>
@@ -2964,7 +3118,13 @@
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Has a SOC policy been created?</t>
+          <t>Has a SOC policy been created?
+Maturity guidance:
+1 - No SOC policy in place
+2 - Some ad-hoc information across documents
+3 - Basic SOC policy document created
+4 - Single document, full description of SOC policy elements
+5 - SOC policy document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3396,13 @@
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Le SOC est-il consulted in the creation and updates of operational security policy?</t>
+          <t>Le SOC est-il consulted in the creation and updates of operational security policy?
+Maturity guidance:
+1 - SOC not consulted or informed of policy creation or policy updates
+2 - SOC informed of policy creation and updates only
+3 - SOC consulted before policy creation and updates, not actively involved
+4 - SOC consulted before policy creation and updates, performs reviews
+5 - Full involvement of the SOC in the creation of operational security policy</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3435,13 @@
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Is a reporting policy for security incidents en place?</t>
+          <t>Is a reporting policy for security incidents en place?
+Maturity guidance:
+1 - No reporting policy in place
+2 - Policy in place, no mention of the SOC
+3 - Policy in place, role of the SOC in security incidents mentioned
+4 - Policy in place with all SOC activities, no central point for reporting
+5 - Policy &amp; central point for reporting in place, SOC part of the workflow</t>
         </is>
       </c>
     </row>
@@ -3302,7 +3474,13 @@
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Is a privacy policy regarding security monitoring of employees en place?</t>
+          <t>Is a privacy policy regarding security monitoring of employees en place?
+Maturity guidance:
+1 - No policy is in place
+2 - Information regarding privacy is scattered across documents
+3 - A policy exists, but has not been accepted formally
+4 - A formal policy exists, its contents are known to all employees
+5 - A formal policy exists, its contents are accepted by all employees</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3513,13 @@
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Le SOC operate in compliance with all applicable privacy laws and regulations?</t>
+          <t>Le SOC operate in compliance with all applicable privacy laws and regulations?
+Maturity guidance:
+1 - Regulations are not known and the SOC is non-compliant
+2 - Some regulations are known and the SOC is non-compliant
+3 - Most regulations are known and the SOC is partially compliant
+4 - Regulations are fully known and the SOC is mostly compliant
+5 - Regulations are fully known and the SOC is fully compliant</t>
         </is>
       </c>
     </row>
@@ -3368,7 +3552,13 @@
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Le SOC cooperate with legal departments regarding privacy matters?</t>
+          <t>Le SOC cooperate with legal departments regarding privacy matters?
+Maturity guidance:
+1 - There is no cooperation between the SOC and legal
+2 - There is some ad-hoc cooperation between SOC and legal
+3 - There is structural cooperation between SOC and legal
+4 - Alignment exists between SOC and legal
+5 - Full and regular alignment exists between SOC and legal</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3591,13 @@
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Are specific procedures en place for dealing with privacy related investigations?</t>
+          <t>Are specific procedures en place for dealing with privacy related investigations?
+Maturity guidance:
+1 - No privacy procedures in place
+2 - Some ad-hoc information across documents
+3 - Basic privacy procedure created
+4 - Single document, full description of privacy investigations
+5 - Procedure completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3630,13 @@
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Is a Privacy Impact Assessment (PIA) regularly conducted?</t>
+          <t>Is a Privacy Impact Assessment (PIA) regularly conducted?
+Maturity guidance:
+1 - PIAs are not conducted
+2 - PIAs are conducted in an ad-hoc fashion
+3 - PIAs are conducted using a structured approach in an ad-hoc fashion
+4 - PIAs are conducted informally and regularly
+5 - PIAs are conducted formally and regularly</t>
         </is>
       </c>
     </row>
@@ -3454,7 +3656,11 @@
         </is>
       </c>
       <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
       <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
@@ -3590,7 +3796,13 @@
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
-          <t>La taille actuelle du SOC du SOC meet les exigences en ETP?</t>
+          <t>La taille actuelle du SOC du SOC meet les exigences en ETP?
+Maturity guidance:
+1 - The SOC is either heavily overstaffed or understaffed
+2 - The SOC is overstaffed or understaffed
+3 - The SOC is somewhat overstaffed or understaffed
+4 - The SOC mostly meets FTE requirements
+5 - The SOC is staffed to full satisfaction in terms of FTE requirements</t>
         </is>
       </c>
     </row>
@@ -3623,7 +3835,13 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Le SOC respecte-t-il les exigences de ratio to external employee le ratio ETP interne/externe?</t>
+          <t>Le SOC respecte-t-il les exigences de ratio to external employee le ratio ETP interne/externe?
+Maturity guidance:
+1 - There are either way too few or too many external employees
+2 - There are too few or too many external employees
+3 - The SOC has somewhat too many or too few external employees
+4 - The SOC mostly meets requirements for external employee FTE count
+5 - The external employee ratio meets all requirements</t>
         </is>
       </c>
     </row>
@@ -3656,7 +3874,13 @@
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Le SOC respecte-t-il les exigences de ratio to external employee skillset?</t>
+          <t>Le SOC respecte-t-il les exigences de ratio to external employee skillset?
+Maturity guidance:
+1 - There are too many skills only present within the external employees
+2 - Some required skills are not present internally, and not transferred
+3 - Some required skills are not present internally, but being transferred
+4 - Most skills are covered with internal employees
+5 - All required skills are covered with internal employees as well</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3913,13 @@
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Tous les postes sont-ils filled?</t>
+          <t>Tous les postes sont-ils filled?
+Maturity guidance:
+1 - Not all positions filled, service delivery cannot be assured
+2 - Sufficient positions filled to ensure service delivery
+3 - All key positions filled
+4 - All positions currently filled, not meeting external ration requirements
+5 - All positions currently filled, meeting external ratio requirements</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3952,13 @@
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Avez-vous un processus de recrutement process en place?</t>
+          <t>Avez-vous un processus de recrutement process en place?
+Maturity guidance:
+1 - There is no recruitment process in place
+2 - Recruitment is performed at an ad-hoc basis
+3 - A basic recruitment process is in place
+4 - A full recruitment process is in place, but not performing effectively
+5 - A full recruitment process is in place and performing effectively</t>
         </is>
       </c>
     </row>
@@ -3755,7 +3991,13 @@
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Avez-vous un processus d'acquisition de talents acquisition process en place?</t>
+          <t>Avez-vous un processus d'acquisition de talents acquisition process en place?
+Maturity guidance:
+1 - No talent acquisition process in place
+2 - Talent acquisition is performed at an ad-hoc basis
+3 - A basic talent acquisition process is in place
+4 - A full acquisition process is in place, but not performing effectively
+5 - A full acquisition process is in place and performing effectively</t>
         </is>
       </c>
     </row>
@@ -3788,7 +4030,13 @@
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Avez-vous des critères spécifiques KSAOs established for le personnel du SOC?</t>
+          <t>Avez-vous des critères spécifiques KSAOs established for le personnel du SOC?
+Maturity guidance:
+1 - KSAOs have not been created
+2 - KSOAs are used ad-hoc in staffing activities
+3 - A basic standardized KSAO set is created
+4 - A full KSAO is created, but not actively used in staffing
+5 - A full KSAO is created, regularly updated and actively used in staffing</t>
         </is>
       </c>
     </row>
@@ -3821,7 +4069,13 @@
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Cherchez-vous activement to create a un environnement psychologiquement sûr pour le personnel du SOC?</t>
+          <t>Cherchez-vous activement to create a un environnement psychologiquement sûr pour le personnel du SOC?
+Maturity guidance:
+1 - A safe environment is not actively created
+2 - Basic awareness of a safe environment exists, but is not implemented
+3 - A safe environment has been established, but not actively managed
+4 - A safe environment has been established, and actively managed
+5 - A safe and actively managed environment exists and is evaluated</t>
         </is>
       </c>
     </row>
@@ -3877,7 +4131,13 @@
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Do you formally differentiate roles withdans le SOC?</t>
+          <t>Do you formally differentiate roles withdans le SOC?
+Maturity guidance:
+1 - No roles are used in the SOC
+2 - Some roles exist, but are not actively being used
+3 - Some roles exist, and are actively being used
+4 - All roles are fully in use, but not formalized
+5 - All roles are fully in use and formalized</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4575,13 @@
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Différenciez-vous tiers within these roles?</t>
+          <t>Différenciez-vous tiers within these roles?
+Maturity guidance:
+1 - No tiers exist within these roles
+2 - Some tiers exist, but are not actively being used
+3 - Some tiers exist, and are actively being used
+4 - All tiers are fully in use, but not formalized
+5 - All relevant roles are tiered and formalized</t>
         </is>
       </c>
     </row>
@@ -4348,7 +4614,13 @@
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Tous les roles sufficiently staffed?</t>
+          <t>Tous les roles sufficiently staffed?
+Maturity guidance:
+1 - None of the roles meets FTE requirements
+2 - Some roles meet FTE requirements
+3 - Vital roles meet FTE requirements
+4 - All vital roles and most other roles meet FTE requirements
+5 - All roles fully meet FTE requirements</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4653,13 @@
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e) role-based hierarchy in your SOC?</t>
+          <t>Y a-t-il un(e) role-based hierarchy in your SOC?
+Maturity guidance:
+1 - No hierarchy exists
+2 - A basic hierarchy exists, but is not fully operational
+3 - A basic hierarchy is in place and fully operational
+4 - A full hierarchy is in place, but not formalized
+5 - A full hierarchy is in place and formalized</t>
         </is>
       </c>
     </row>
@@ -4414,7 +4692,13 @@
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
-          <t>Avez-vous formellement documented all SOC roles?</t>
+          <t>Avez-vous formellement documented all SOC roles?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of SOC roles
+4 - Single document, full description of SOC roles
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -4686,7 +4970,13 @@
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
         <is>
-          <t>Are responsibilities for each role understood?</t>
+          <t>Are responsibilities for each role understood?
+Maturity guidance:
+1 - Responsibilities not understood
+2 - Basic awareness of responsibilities
+3 - Responsibilities for some roles understood and adhered to
+4 - Responsibilities for all roles mostly understood and adhered to
+5 - Full understanding of responsibilities formalized in training sessions</t>
         </is>
       </c>
     </row>
@@ -4719,7 +5009,13 @@
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Avez-vous documenté career progression requirements for each of these roles?</t>
+          <t>Avez-vous documenté career progression requirements for each of these roles?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of career progression for roles
+4 - Single document, full description of career progression for roles
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -4752,7 +5048,13 @@
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Effectuez-vous régulièrement revise or update the role descriptions?</t>
+          <t>Effectuez-vous régulièrement revise or update the role descriptions?
+Maturity guidance:
+1 - Documentation is not reviewed
+2 - Documentation is reviewed ad-hoc, not using a structured approach
+3 - Documentation is reviewed ad-hoc, using a structured approach
+4 - Documentation is regularly and informally reviewed and updated
+5 - Documentation is regularly and formally reviewed and updated</t>
         </is>
       </c>
     </row>
@@ -4808,7 +5110,13 @@
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) job rotation plan en place?</t>
+          <t>Avez-vous un(e) job rotation plan en place?
+Maturity guidance:
+1 - No plan exists
+2 - A plan covering some roles is in place, but not operational
+3 - A plan covering some roles is in place and operational
+4 - A plan covering all roles is in place, but not formalized
+5 - A plan covering all roles is in place and formalized</t>
         </is>
       </c>
     </row>
@@ -4841,7 +5149,13 @@
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) career progression process en place?</t>
+          <t>Avez-vous un(e) career progression process en place?
+Maturity guidance:
+1 - No career progression process is in place
+2 - A process covering some roles is in place, but not operational
+3 - A process covering some roles is in place and operational
+4 - A process covering all roles is in place, but not formalized
+5 - A process covering all roles is in place and formalized</t>
         </is>
       </c>
     </row>
@@ -4874,7 +5188,13 @@
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Avez-vous un processus d'acquisition de talents management process en place?</t>
+          <t>Avez-vous un processus d'acquisition de talents management process en place?
+Maturity guidance:
+1 - No talent management process in place
+2 - Talent management is performed at an ad-hoc basis
+3 - A basic talent management process is in place
+4 - A full process is in place, but not performing effectively
+5 - A full talent management process is in place and performing effectively</t>
         </is>
       </c>
     </row>
@@ -4907,7 +5227,13 @@
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Do you have team diversity goals?</t>
+          <t>Do you have team diversity goals?
+Maturity guidance:
+1 - No diversity goals exist
+2 - Diversity goals are recognized but not defined
+3 - Diversity goals are defined but not formalized
+4 - Diversity goals have been formally defined and are not met
+5 - Diversity goals have been formally defined and are met</t>
         </is>
       </c>
     </row>
@@ -4940,7 +5266,13 @@
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Avez-vous établi team goals?</t>
+          <t>Avez-vous établi team goals?
+Maturity guidance:
+1 - Team goals are not determined
+2 - Team goals are determined, but not formally documented
+3 - Team goals are determined, and formally documented
+4 - Team goals are determined and documented, but not tracked
+5 - Team goals are determined, approved and tracked regularly</t>
         </is>
       </c>
     </row>
@@ -4973,7 +5305,13 @@
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Do you document and track individual team member goals?</t>
+          <t>Do you document and track individual team member goals?
+Maturity guidance:
+1 - Individual goals are not determined
+2 - Individual goals are determined, but not formally documented
+3 - Individual goals are determined, and formally documented
+4 - Individual goals are determined and documented, but not tracked
+5 - Individual goals are determined, approved and tracked regularly</t>
         </is>
       </c>
     </row>
@@ -5006,7 +5344,13 @@
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
         <is>
-          <t>Do you periodically evaluate les employés du SOC?</t>
+          <t>Do you periodically evaluate les employés du SOC?
+Maturity guidance:
+1 - No periodic evaluation is performed
+2 - Periodic evaluation is performed in an ad-hoc fashion
+3 - Periodic evaluation is performed in a structured fashion
+4 - Periodic evaluation is performed, but results are not used structurally
+5 - Periodic evaluation is performed, results are used for personal growth</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5383,13 @@
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) 'new hire' process en place?</t>
+          <t>Avez-vous un(e) 'new hire' process en place?
+Maturity guidance:
+1 - No new hire process in place
+2 - New hire training is done in an ad-hoc fashion
+3 - A process is in place, but does not cover all aspects
+4 - An informal process covering people, process and technology is in place
+5 - A formal process covering people, process and technology is in place</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5422,13 @@
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Tous les cas d'usage du SOC sont-ils employees subjected to screening?</t>
+          <t>Tous les cas d'usage du SOC sont-ils employees subjected to screening?
+Maturity guidance:
+1 - Screening not performed
+2 - Basic screening performed in ad-hoc fashion
+3 - Basic screening procedure in place, applied structurally
+4 - Full screening procedure in place, applied structurally, not formalized
+5 - Formal screening procedure and background checks applied structurally</t>
         </is>
       </c>
     </row>
@@ -5105,7 +5461,13 @@
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Mesurez-vous employee satisfaction for improving le SOC?</t>
+          <t>Mesurez-vous employee satisfaction for improving le SOC?
+Maturity guidance:
+1 - Employee satisfaction is not measured
+2 - Employee satisfaction is measured in an ad-hoc fashion
+3 - Satisfaction is usually measured, but not embedded in processes
+4 - Employee satisfaction is measured, not used for improvement
+5 - Employee satisfaction measured periodically and used for improvement</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5500,13 @@
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Y a-t-il regular 1-on-1 meetings between le SOC manager and the employees?</t>
+          <t>Y a-t-il regular 1-on-1 meetings between le SOC manager and the employees?
+Maturity guidance:
+1 - 1-on-1 meetings are not held within the SOC
+2 - 1-on-1 meetings are held on ad-hoc basis
+3 - Informal 1-on-1 meetings are held periodically
+4 - Formal 1-on-1 meetings are regularly held, results are not structured
+5 - 1-on-1 meetings are regularly held and used for coaching and growth</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5539,13 @@
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Effectuez-vous regular teambuilding exercises?</t>
+          <t>Effectuez-vous regular teambuilding exercises?
+Maturity guidance:
+1 - No team building exercises are performed
+2 - Exercises are performed in an ad-hoc fashion
+3 - Exercises are usually performed, but not embedded in processes
+4 - Exercises are regularly done, but not focused on improvement
+5 - Exercises are regularly done and focused on improving team dynamics</t>
         </is>
       </c>
     </row>
@@ -5204,7 +5578,13 @@
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
         <is>
-          <t>Effectuez-vous regular teambuilding exercises with other teams relevant to le SOC?</t>
+          <t>Effectuez-vous regular teambuilding exercises with other teams relevant to le SOC?
+Maturity guidance:
+1 - No MTS team building exercises are performed
+2 - MTS exercises are performed in an ad-hoc fashion
+3 - MTS exercises are usually performed, but not embedded in processes
+4 - MTS exercises are regularly done, but not focused on improvement
+5 - MTS exercises done regularly and focused on improving team dynamics</t>
         </is>
       </c>
     </row>
@@ -5237,7 +5617,13 @@
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
-          <t>Do you periodically evaluate team performance?</t>
+          <t>Do you periodically evaluate team performance?
+Maturity guidance:
+1 - No periodic evaluation is performed
+2 - Periodic evaluation is performed in an ad-hoc fashion
+3 - Periodic evaluation is performed in a structured fashion
+4 - Periodic evaluation is performed, but results are not used structurally
+5 - Periodic evaluation is performed, results are used for team growth</t>
         </is>
       </c>
     </row>
@@ -5293,7 +5679,13 @@
       <c r="F157" t="inlineStr"/>
       <c r="G157" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) formal knowledge management process en place?</t>
+          <t>Avez-vous un(e) formal knowledge management process en place?
+Maturity guidance:
+1 - A knowledge management process is not in place
+2 - Knowledge management is done in an ad-hoc fashion
+3 - A basic process is in place, that covers some knowledge aspects
+4 - An informal process is in place that covers most knowledge aspects
+5 - A formal process is in place, covering all knowledge aspects</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5718,13 @@
       <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) skill matrix en place?</t>
+          <t>Avez-vous un(e) skill matrix en place?
+Maturity guidance:
+1 - A skill matrix is not in place
+2 - A basic skill matrix is in place, but incomplete
+3 - A complete skill matrix is in place, not approved
+4 - A complete skill matrix is in place and approved, not regularly updated
+5 - A complete skill matrix is in place, approved and regularly updated</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5888,13 @@
       <c r="F164" t="inlineStr"/>
       <c r="G164" t="inlineStr">
         <is>
-          <t>Is the skill matrix actively used for team and personal improvement?</t>
+          <t>Is the skill matrix actively used for team and personal improvement?
+Maturity guidance:
+1 - Matrix not used for improvement
+2 - Matrix used for improvement in an ad-hoc fashion
+3 - Matrix used to improve some personal and team results
+4 - Matrix used to improve all personal and team results
+5 - Matrix used to improve personal and team results, improvements tracked</t>
         </is>
       </c>
     </row>
@@ -5523,7 +5927,13 @@
       <c r="F165" t="inlineStr"/>
       <c r="G165" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) knowledge matrix en place?</t>
+          <t>Avez-vous un(e) knowledge matrix en place?
+Maturity guidance:
+1 - A knowledge matrix is not in place
+2 - A basic knowledge matrix is in place, but incomplete
+3 - A complete knowledge matrix is in place, not approved
+4 - A complete knowledge matrix is in place and approved, not regularly updated
+5 - A complete knowledge matrix is in place, approved and regularly updated</t>
         </is>
       </c>
     </row>
@@ -5660,7 +6070,13 @@
       <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
-          <t>Is the knowledge matrix actively used to determine training and education needs?</t>
+          <t>Is the knowledge matrix actively used to determine training and education needs?
+Maturity guidance:
+1 - Matrix not used for identification of training needs
+2 - Matrix used for training identification in an ad-hoc fashion
+3 - Matrix used to identify training needs, but not for all employees
+4 - Matrix used to identify all training needs, but not tracked for execution
+5 - Matrix structurally used to identify training needs, training tracked</t>
         </is>
       </c>
     </row>
@@ -5693,7 +6109,13 @@
       <c r="F171" t="inlineStr"/>
       <c r="G171" t="inlineStr">
         <is>
-          <t>Avez-vous documenté SOC team member abilities?</t>
+          <t>Avez-vous documenté SOC team member abilities?
+Maturity guidance:
+1 - Documentation is not in place
+2 - Documentation only covers some employees' abilities
+3 - Documentation covers the most relevant abilities for the team
+4 - All employee abilities documented, but is not regularly updated
+5 - All employee abilities documented, and regularly updated</t>
         </is>
       </c>
     </row>
@@ -5726,7 +6148,13 @@
       <c r="F172" t="inlineStr"/>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Effectuez-vous régulièrement assess and revise the knowledge management process?</t>
+          <t>Effectuez-vous régulièrement assess and revise the knowledge management process?
+Maturity guidance:
+1 - Documentation is not reviewed
+2 - Documentation is reviewed ad-hoc, not using a structured approach
+3 - Documentation is reviewed ad-hoc, using a structured approach
+4 - Documentation is regularly and informally reviewed and updated
+5 - Documentation is regularly and formally reviewed and updated</t>
         </is>
       </c>
     </row>
@@ -5759,7 +6187,13 @@
       <c r="F173" t="inlineStr"/>
       <c r="G173" t="inlineStr">
         <is>
-          <t>Existe-t-il effective tooling en place to support knowledge documentation and distribution?</t>
+          <t>Existe-t-il effective tooling en place to support knowledge documentation and distribution?
+Maturity guidance:
+1 - Tooling is not in place
+2 - Tooling is in place, but used in an ad-hoc fashion
+3 - Tooling is in place, and used regularly
+4 - Tooling is in place and use of the tool is embedded in processes
+5 - Tooling is in place and optimized for knowledge management purposes</t>
         </is>
       </c>
     </row>
@@ -5815,7 +6249,13 @@
       <c r="F175" t="inlineStr"/>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) training program en place?</t>
+          <t>Avez-vous un(e) training program en place?
+Maturity guidance:
+1 - A training program is not in place
+2 - A training program some roles is in place, but not operational
+3 - A training program covering some roles is in place and operational
+4 - A training program covering all roles is in place, but not formalized
+5 - A training program covering all roles is in place and formalized</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6473,13 @@
       <c r="F183" t="inlineStr"/>
       <c r="G183" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) certification program en place?</t>
+          <t>Avez-vous un(e) certification program en place?
+Maturity guidance:
+1 - A certification program is not in place
+2 - A certification program some roles is in place, but not operational
+3 - A certification program covering some roles is in place and operational
+4 - A certification program covering all roles is in place, but not formalized
+5 - A certification program covering all roles is in place and formalized</t>
         </is>
       </c>
     </row>
@@ -6170,7 +6616,13 @@
       <c r="F188" t="inlineStr"/>
       <c r="G188" t="inlineStr">
         <is>
-          <t>Is the training and certification program connected to evaluation and career progression?</t>
+          <t>Is the training and certification program connected to evaluation and career progression?
+Maturity guidance:
+1 - The programs are not connected
+2 - The programs are connected in an ad-hoc fashion
+3 - The programs are regularly used, but not embedded in processes
+4 - The programs are mostly aligned, but not formally
+5 - The programs are formally embedded in evaluation and progression</t>
         </is>
       </c>
     </row>
@@ -6203,7 +6655,13 @@
       <c r="F189" t="inlineStr"/>
       <c r="G189" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e) reserved budget for education and training?</t>
+          <t>Y a-t-il un(e) reserved budget for education and training?
+Maturity guidance:
+1 - No budget is allocated
+2 - Insufficient budget is allocated for the team as a whole
+3 - Sufficient budget is allocated for the team as a whole
+4 - Employees have sufficient budget, not encouraged to attend training
+5 - Employees have sufficient budget, encouraged to attend training</t>
         </is>
       </c>
     </row>
@@ -6236,7 +6694,13 @@
       <c r="F190" t="inlineStr"/>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e) reserved amount of time for education and training?</t>
+          <t>Y a-t-il un(e) reserved amount of time for education and training?
+Maturity guidance:
+1 - No time is allocated
+2 - Insufficient time is allocated for the team as a whole
+3 - Sufficient time is allocated for the team as a whole
+4 - Employees have sufficient time, but not encouraged to attend training
+5 - Employees have sufficient time, and encouraged to attend training</t>
         </is>
       </c>
     </row>
@@ -6269,7 +6733,13 @@
       <c r="F191" t="inlineStr"/>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Do you have regular workshops for knowledge development?</t>
+          <t>Do you have regular workshops for knowledge development?
+Maturity guidance:
+1 - Workshops are not held
+2 - Workshops are held in an ad-hoc fashion
+3 - Workshops are held periodically
+4 - Workshops are held regularly, not aligned with knowledge &amp; training
+5 - Workshops are held regularly and aligned with knowledge &amp; training</t>
         </is>
       </c>
     </row>
@@ -6302,7 +6772,13 @@
       <c r="F192" t="inlineStr"/>
       <c r="G192" t="inlineStr">
         <is>
-          <t>Effectuez-vous régulièrement revise and update the training and certification programs?</t>
+          <t>Effectuez-vous régulièrement revise and update the training and certification programs?
+Maturity guidance:
+1 - Programs are not reviewed
+2 - Programs are reviewed ad-hoc, not using a structured approach
+3 - Programs are reviewed ad-hoc, using a structured approach
+4 - Programs are regularly and informally reviewed and updated
+5 - Programs are regularly and formally reviewed and updated</t>
         </is>
       </c>
     </row>
@@ -6322,7 +6798,11 @@
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
-      <c r="F193" t="inlineStr"/>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
       <c r="G193" t="inlineStr"/>
     </row>
     <row r="194">
@@ -6377,7 +6857,13 @@
       <c r="F195" t="inlineStr"/>
       <c r="G195" t="inlineStr">
         <is>
-          <t>Y a-t-il un SOC management process en place?</t>
+          <t>Y a-t-il un SOC management process en place?
+Maturity guidance:
+1 - A SOC management process is not in place
+2 - SOC management is done in an ad-hoc fashion
+3 - A basic process is in place, that covers some aspects
+4 - An informal process is in place that covers most aspects
+5 - A formal process is in place, covering all aspects</t>
         </is>
       </c>
     </row>
@@ -6410,7 +6896,13 @@
       <c r="F196" t="inlineStr"/>
       <c r="G196" t="inlineStr">
         <is>
-          <t>Les éléments de gestion du SOC sont-ils elements formellement identifiés et documentés?</t>
+          <t>Les éléments de gestion du SOC sont-ils elements formellement identifiés et documentés?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of SOC management process
+4 - Single document, full description of SOC management process
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -6736,7 +7228,13 @@
       <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
-          <t>Le processus de gestion du SOC est-il process régulièrement revu?</t>
+          <t>Le processus de gestion du SOC est-il process régulièrement revu?
+Maturity guidance:
+1 - SOC management process is not reviewed
+2 - SOC management process is reviewed in an ad-hoc fashion
+3 - Process is reviewed using a structured approach in an ad-hoc fashion
+4 - Process is regularly and informally reviewed and updated
+5 - Process is regularly and formally reviewed and updated with findings</t>
         </is>
       </c>
     </row>
@@ -6769,7 +7267,13 @@
       <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Le processus de gestion du SOC est-il process aligné avec toutes les parties prenantes?</t>
+          <t>Le processus de gestion du SOC est-il process aligné avec toutes les parties prenantes?
+Maturity guidance:
+1 - Stakeholders are unfamiliar with the process
+2 - Some stakeholders are aware of the process, but not its details
+3 - Some stakeholders are aware of the process and its details
+4 - All stakeholders are aware, not all stakeholders know its details
+5 - All stakeholders are aware of the process and its details</t>
         </is>
       </c>
     </row>
@@ -6802,7 +7306,13 @@
       <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
-          <t>Avez-vous mis en place un processus d'amélioration continue (CI)?</t>
+          <t>Avez-vous mis en place un processus d'amélioration continue (CI)?
+Maturity guidance:
+1 - CI process not implemented
+2 - CI conducted in an ad-hoc fashion
+3 - CI conducted structurally, not documented
+4 - CI conducted structurally, following a defined process
+5 - CI conducted structurally, following an approved and measured process</t>
         </is>
       </c>
     </row>
@@ -7286,7 +7796,13 @@
       <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
-          <t>Avez-vous mis en place un processus d'architecture SOC?</t>
+          <t>Avez-vous mis en place un processus d'architecture SOC?
+Maturity guidance:
+1 - Architecture process not in place
+2 - Architecture conducted in an ad-hoc fashion
+3 - Basic documentation of SOC architecture, principles defined
+4 - SOC architecture process completed, not used consistently decisions
+5 - SOC architecture process approved and used actively in decision making</t>
         </is>
       </c>
     </row>
@@ -7527,7 +8043,13 @@
       <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) documented exercise plan?</t>
+          <t>Avez-vous un(e) documented exercise plan?
+Maturity guidance:
+1 - No exercise plan in place
+2 - Some ad-hoc information across documents
+3 - Basic description of SOC exercises
+4 - Single document, full description of SOC exercises
+5 - Exercises plan completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -7745,7 +8267,13 @@
       <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
-          <t>Effectuez-vous les opérations de sécurité exercises regularly?</t>
+          <t>Effectuez-vous les opérations de sécurité exercises regularly?
+Maturity guidance:
+1 - No security operations exercises are performed
+2 - Exercises are performed on ad-hoc basis
+3 - Exercises are sometimes performed in a structured manner
+4 - Informal structured exercises are performed regularly
+5 - Formal structured exercises are performed regularly</t>
         </is>
       </c>
     </row>
@@ -7778,7 +8306,13 @@
       <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
-          <t>Are the results from exercises documented?</t>
+          <t>Are the results from exercises documented?
+Maturity guidance:
+1 - Results not documented
+2 - Results documented in a ad-hoc fashion
+3 - Results documented in a single document
+4 - Results documented using a defined template
+5 - Results documented, reviewed and formally approved</t>
         </is>
       </c>
     </row>
@@ -7811,7 +8345,13 @@
       <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
-          <t>Is the output from exercises actively used to improve les opérations de sécurité?</t>
+          <t>Is the output from exercises actively used to improve les opérations de sécurité?
+Maturity guidance:
+1 - Output not used for improvement purposes
+2 - Improvements done in an ad-hoc fashion
+3 - Improvements determined and documented
+4 - Improvements determined and formally approved
+5 - Improvements determined, formally assigned, implementation tracked</t>
         </is>
       </c>
     </row>
@@ -7871,7 +8411,13 @@
       <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
-          <t>Do you have standard operating procedures?</t>
+          <t>Do you have standard operating procedures?
+Maturity guidance:
+1 - No standard operating procedures are in place
+2 - Only vital procedures are in place
+3 - Most procedures are in place
+4 - All procedures are in place, not optimized through feedback
+5 - All procedures are in place, up to date and optimized for performance</t>
         </is>
       </c>
     </row>
@@ -7904,7 +8450,13 @@
       <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
-          <t>Utilisez-vous checklists for recurring activities?</t>
+          <t>Utilisez-vous checklists for recurring activities?
+Maturity guidance:
+1 - No checklists are in place
+2 - A basic checklist is used in an ad-hoc fashion
+3 - Checklists are in place, but not used consistently
+4 - Checklists are used consistently, but not formally signed off
+5 - Checklists are used consistently and formally signed off</t>
         </is>
       </c>
     </row>
@@ -7937,7 +8489,13 @@
       <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
-          <t>Utilisez-vous documented workflows?</t>
+          <t>Utilisez-vous documented workflows?
+Maturity guidance:
+1 - Workflows are not in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of workflows
+4 - Single document, full description of workflows
+5 - Workflows are completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -7970,7 +8528,13 @@
       <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
-          <t>Avez-vous un SOC operational handbook?</t>
+          <t>Avez-vous un SOC operational handbook?
+Maturity guidance:
+1 - An operational handbook is not in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of SOC tasks &amp; rules
+4 - Single document, full description of SOC tasks &amp; rules
+5 - Handbook is completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -8003,7 +8567,13 @@
       <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
-          <t>Avez-vous établi an Operational Security (OPSEC) program?</t>
+          <t>Avez-vous établi an Operational Security (OPSEC) program?
+Maturity guidance:
+1 - An OPSEC program is not in place
+2 - Some ad-hoc information across documents regarding OPSEC
+3 - Consistent OPSEC documentation, no program
+4 - Comprehensive OPSEC program exists, not consistently enforced/maintained
+5 - OPSEC program is formally approved, enforced and regularly maintained</t>
         </is>
       </c>
     </row>
@@ -8063,7 +8633,13 @@
       <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
-          <t>Are ITSM processes integrated dans le SOC?</t>
+          <t>Are ITSM processes integrated dans le SOC?
+Maturity guidance:
+1 - ITSM processes not integrated
+2 - ITSM process integrations performed in an ad-hoc fashion
+3 - ITSM process integrations in place, not structurally executed
+4 - ITSM process integrations in place, structurally executed
+5 - ITSM processes integrated, executed, and optimized</t>
         </is>
       </c>
     </row>
@@ -8254,7 +8830,13 @@
       <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
-          <t>Are ITSM processes integrations regularly evaluated?</t>
+          <t>Are ITSM processes integrations regularly evaluated?
+Maturity guidance:
+1 - ITSM processes integrations not evaluated
+2 - ITSM process integrations evaluated in an ad-hoc fashion
+3 - ITSM process integration evaluation in place, not structurally executed
+4 - ITSM process integration evaluation in place, structurally executed
+5 - ITSM processes integration evaluation in place, aligned with stakeholders</t>
         </is>
       </c>
     </row>
@@ -8314,7 +8896,13 @@
       <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) dedicated physical SOC location?</t>
+          <t>Avez-vous un(e) dedicated physical SOC location?
+Maturity guidance:
+1 - No dedicated physical location
+2 - Floorplan in place, not operationalized
+3 - SOC established on single floor, some facilities in place
+4 - Dedicated location established, most facilities in place
+5 - Dedicated secure location established, fully optimized for sec ops</t>
         </is>
       </c>
     </row>
@@ -8613,7 +9201,13 @@
       <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
-          <t>Avez-vous mis en place shifts dans le SOC?</t>
+          <t>Avez-vous mis en place shifts dans le SOC?
+Maturity guidance:
+1 - Shift schedules not in place
+2 - Basic schedule in place, not applied structurally
+3 - Basic schedule in place, applied structurally
+4 - Shift schedules in place, covering most requirements
+5 - Shift schedules in place, covering all requirements with full coverage</t>
         </is>
       </c>
     </row>
@@ -8646,7 +9240,13 @@
       <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
-          <t>Have schedules been optimized for vigilance during shifts?</t>
+          <t>Have schedules been optimized for vigilance during shifts?
+Maturity guidance:
+1 - Shift schedules not created with vigilance in mind
+2 - Vigilance requirements understood, but not implemented
+3 - Vigilance requirements implemented, but not optimized
+4 - Shift schedule optimized for vigilance, but not regularly improved
+5 - Shift schedule optimized for vigilance, regularly evaluated and improved</t>
         </is>
       </c>
     </row>
@@ -8895,7 +9495,13 @@
       <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) Document Management System en place?</t>
+          <t>Avez-vous un(e) Document Management System en place?
+Maturity guidance:
+1 - No DMS in place
+2 - Documentation centralized on file shares
+3 - DMS in place, documentation updates not enforced
+4 - DMS in place, documentation updates and versions enforced
+5 - DMS in place, fully supporting SOC documentation requirements</t>
         </is>
       </c>
     </row>
@@ -8928,7 +9534,13 @@
       <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
         <is>
-          <t>Avez-vous un(e) knowledge &amp; collaboration platform en place?</t>
+          <t>Avez-vous un(e) knowledge &amp; collaboration platform en place?
+Maturity guidance:
+1 - No knowledge &amp; collaboration platform in place
+2 - Knowledge &amp; collaboration performed in an ad-hoc fashion
+3 - Platform in place, not dedicated, not restricted to SOC
+4 - Platform in place, not dedicated, restricted to SOC
+5 - Dedicated platform, fully supporting sec ops, integrated in ITSM process</t>
         </is>
       </c>
     </row>
@@ -8984,7 +9596,13 @@
       <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Reports</t>
+          <t>Reports
+Maturity guidance:
+1 - No reports are provided
+2 - Reports are provided in an ad-hoc fashion
+3 - Reports are provided regularly, not standardized
+4 - Reports are provided regularly and standardized using quality criteria
+5 - Reports are provided regularly, standardized and regularly optimized</t>
         </is>
       </c>
     </row>
@@ -9445,7 +10063,13 @@
       <c r="F305" t="inlineStr"/>
       <c r="G305" t="inlineStr">
         <is>
-          <t>Métriques</t>
+          <t>Métriques
+Maturity guidance:
+1 - Reports not tailored
+2 - Only basic customizations for customers applied
+3 - Customizations applied structurally to customer reports
+4 - Reports fully tailored to recipients, manual customization required
+5 - Reports fully tailored to recipients using automated templates</t>
         </is>
       </c>
     </row>
@@ -9690,7 +10314,13 @@
       <c r="F314" t="inlineStr"/>
       <c r="G314" t="inlineStr">
         <is>
-          <t>Advisories</t>
+          <t>Advisories
+Maturity guidance:
+1 - Reports not approved or reviewed
+2 - Informal report review conducted
+3 - Structural report review conducted
+4 - Reports regularly reviewed, not formally signed off by recipients
+5 - Reports regularly reviewed and formally signed off by recipients</t>
         </is>
       </c>
     </row>
@@ -9804,7 +10434,13 @@
       <c r="F318" t="inlineStr"/>
       <c r="G318" t="inlineStr">
         <is>
-          <t>Education and Awareness</t>
+          <t>Education and Awareness
+Maturity guidance:
+1 - No established reporting lines
+2 - Reports have limited dissemination
+3 - Reports have a standard distribution list
+4 - Reports dissemination through standard reporting lines, not approved
+5 - Reports dissemination through standard and approved reporting lines</t>
         </is>
       </c>
     </row>
@@ -9891,7 +10527,13 @@
       <c r="F321" t="inlineStr"/>
       <c r="G321" t="inlineStr">
         <is>
-          <t>Communication</t>
+          <t>Communication
+Maturity guidance:
+1 - Report templates not updated
+2 - Report templates updated in an ad-hoc fashion
+3 - Report templates regularly revised and updated
+4 - Report templates revised and updated using customer feedback
+5 - Reports templates regularly updated and formally approved</t>
         </is>
       </c>
     </row>
@@ -10036,9 +10678,17 @@
           <t>Process.4.1</t>
         </is>
       </c>
-      <c r="D327" t="inlineStr"/>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>[Process.4.1]</t>
+        </is>
+      </c>
       <c r="E327" t="inlineStr"/>
-      <c r="F327" t="inlineStr"/>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>[Process.4.1]</t>
+        </is>
+      </c>
       <c r="G327" t="inlineStr"/>
     </row>
     <row r="328">
@@ -10348,9 +10998,17 @@
           <t>Process.4.2</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr"/>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>[Process.4.2]</t>
+        </is>
+      </c>
       <c r="E339" t="inlineStr"/>
-      <c r="F339" t="inlineStr"/>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>[Process.4.2]</t>
+        </is>
+      </c>
       <c r="G339" t="inlineStr"/>
     </row>
     <row r="340">
@@ -10382,7 +11040,13 @@
       <c r="F340" t="inlineStr"/>
       <c r="G340" t="inlineStr">
         <is>
-          <t>Mesurez-vous les cas d'usage par rapport au référentiel MITRE ATT&amp;CK® à des fins d'analyse des écarts?</t>
+          <t>Mesurez-vous les cas d'usage par rapport au référentiel MITRE ATT&amp;CK® à des fins d'analyse des écarts?
+Maturity guidance:
+1 - Use cases not measured against Mitre ATT&amp;CK
+2 - High risk use cases measured against MITRE ATT&amp;CK®
+3 - High- and medium risk use cases measured against MITRE ATT&amp;CK®
+4 - All use cases frequently measured, output used in improvement
+5 - All use cases continuously measured, output used in improvement</t>
         </is>
       </c>
     </row>
@@ -10415,7 +11079,13 @@
       <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
-          <t>Les règles de surveillance sont-elles tagged with les identifiants du référentiel MITRE ATT&amp;CK®? [2]</t>
+          <t>Les règles de surveillance sont-elles tagged with les identifiants du référentiel MITRE ATT&amp;CK®? [2]
+Maturity guidance:
+1 - Monitoring rules not tagged
+2 - High risk monitoring rules tagged
+3 - High- and medium risk monitoring rules tagged
+4 - All monitoring rules tagged, not regularly revised
+5 - All monitoring rules tagged and regularly revised</t>
         </is>
       </c>
     </row>
@@ -10448,7 +11118,13 @@
       <c r="F342" t="inlineStr"/>
       <c r="G342" t="inlineStr">
         <is>
-          <t>Avez-vous créé un profil de risque MITRE ATT&amp;CK® pour votre organisation?</t>
+          <t>Avez-vous créé un profil de risque MITRE ATT&amp;CK® pour votre organisation?
+Maturity guidance:
+1 - MITRE ATT&amp;CK® profile not created
+2 - MITRE ATT&amp;CK® analysis performed, no formal profile in place
+3 - MITRE ATT&amp;CK® profile created, not validated or maintained
+4 - MITRE ATT&amp;CK® profile created and validated, not regularly maintained
+5 - Mitre ATT&amp;CK profile created, validated and regularly maintained</t>
         </is>
       </c>
     </row>
@@ -10481,7 +11157,13 @@
       <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr">
         <is>
-          <t>Avez-vous priorisé les techniques MITRE ATT&amp;CK® selon la pertinence? [3]</t>
+          <t>Avez-vous priorisé les techniques MITRE ATT&amp;CK® selon la pertinence? [3]
+Maturity guidance:
+1 - ATT&amp;CK® techniques not prioritized
+2 - ATT&amp;CK® analysis performed, no formal prioritization created
+3 - ATT&amp;CK® techniques prioritized, not validated or maintained
+4 - ATT&amp;CK® techniques prioritized and validated, not regularly maintained
+5 - ATT&amp;CK® techniques prioritized, validated and regularly updated</t>
         </is>
       </c>
     </row>
@@ -10514,7 +11196,13 @@
       <c r="F344" t="inlineStr"/>
       <c r="G344" t="inlineStr">
         <is>
-          <t>La sortie des cas d'usage est-elle output (alerts) utilisé dans les activités de renseignement sur les menaces?</t>
+          <t>La sortie des cas d'usage est-elle output (alerts) utilisé dans les activités de renseignement sur les menaces?
+Maturity guidance:
+1 - Use case output not used in TI activities
+2 - Use case output used in TI activities in an ad-hoc fashion
+3 - Use case output used in TI activities for high-risk alerts
+4 - Use case output used in TI activities for most alerts, no formal process
+5 - Formal process in place, connecting use case output to TI activities</t>
         </is>
       </c>
     </row>
@@ -10547,7 +11235,13 @@
       <c r="F345" t="inlineStr"/>
       <c r="G345" t="inlineStr">
         <is>
-          <t>Is threat intelligence used for the creation and updates of use cases?</t>
+          <t>Is threat intelligence used for the creation and updates of use cases?
+Maturity guidance:
+1 - TI not used in use case creation / updates
+2 - TI used in use case creation / updates in an ad-hoc fashion
+3 - TI used in use case creation / updates for high-risk threats
+4 - TI used in use case creation / updates for most threats, no formal process
+5 - Formal process in place, connecting TI activities to use cases</t>
         </is>
       </c>
     </row>
@@ -10561,9 +11255,17 @@
           <t>Process.4.3</t>
         </is>
       </c>
-      <c r="D346" t="inlineStr"/>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>[Process.4.3]</t>
+        </is>
+      </c>
       <c r="E346" t="inlineStr"/>
-      <c r="F346" t="inlineStr"/>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>[Process.4.3]</t>
+        </is>
+      </c>
       <c r="G346" t="inlineStr"/>
     </row>
     <row r="347">
@@ -10595,7 +11297,13 @@
       <c r="F347" t="inlineStr"/>
       <c r="G347" t="inlineStr">
         <is>
-          <t>Déterminez-vous and document visibility requirements for each use case?</t>
+          <t>Déterminez-vous and document visibility requirements for each use case?
+Maturity guidance:
+1 - Visibility requirements not determined
+2 - Visibility requirements determined for some use cases
+3 - Visibility requirements determined for most use cases, not documented
+4 - Visibility requirements formally determined and documented, not reviewed
+5 - Visibility requirements formally determined, documented and reviewed</t>
         </is>
       </c>
     </row>
@@ -10628,7 +11336,13 @@
       <c r="F348" t="inlineStr"/>
       <c r="G348" t="inlineStr">
         <is>
-          <t>Mesurez-vous la visibilité status pour vos cas d'usage à des fins d'analyse des écarts?</t>
+          <t>Mesurez-vous la visibilité status pour vos cas d'usage à des fins d'analyse des écarts?
+Maturity guidance:
+1 - Visibility status not measured
+2 - Visibility status measured in an ad-hoc fashion
+3 - Visibility status measured, not actively used in improvement
+4 - Visibility status measured frequently, output used in improvement
+5 - Visibility status continuously measured, output used in improvement</t>
         </is>
       </c>
     </row>
@@ -10661,7 +11375,13 @@
       <c r="F349" t="inlineStr"/>
       <c r="G349" t="inlineStr">
         <is>
-          <t>Mappez-vous les sources de données source visibility to the le référentiel MITRE ATT&amp;CK®? [4]</t>
+          <t>Mappez-vous les sources de données source visibility to the le référentiel MITRE ATT&amp;CK®? [4]
+Maturity guidance:
+1 - Data sources not mapped to MITRE ATT&amp;CK®
+2 - Data source mapping to ATT&amp;CK® performed in an ad-hoc fashion
+3 - Data sources mapped to ATT&amp;CK®, not actively used in improvement
+4 - Data sources frequently mapped to ATT&amp;CK®, output used in improvement
+5 - Data sources continuously mapped to ATT&amp;CK®, output used in improvement</t>
         </is>
       </c>
     </row>
@@ -10698,9 +11418,17 @@
           <t>Process.5.1</t>
         </is>
       </c>
-      <c r="D351" t="inlineStr"/>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>[Process.5.1]</t>
+        </is>
+      </c>
       <c r="E351" t="inlineStr"/>
-      <c r="F351" t="inlineStr"/>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>[Process.5.1]</t>
+        </is>
+      </c>
       <c r="G351" t="inlineStr"/>
     </row>
     <row r="352">
@@ -10732,7 +11460,13 @@
       <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
-          <t>Avez-vous un processus de détection engineering process en place?</t>
+          <t>Avez-vous un processus de détection engineering process en place?
+Maturity guidance:
+1 - A detection engineering process is not in place
+2 - Detection engineering is done in an ad-hoc fashion
+3 - Basic process in place, not applied to all use cases
+4 - Informal process in place covering all use cases
+5 - Formal process in place, covering all use cases</t>
         </is>
       </c>
     </row>
@@ -10765,7 +11499,13 @@
       <c r="F353" t="inlineStr"/>
       <c r="G353" t="inlineStr">
         <is>
-          <t>La détection est-elle engineering process formellement documenté?</t>
+          <t>La détection est-elle engineering process formellement documenté?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of detection engineering process
+4 - Single document, full description of detection engineering process
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -10798,7 +11538,13 @@
       <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
-          <t>Y a-t-il des rôles spécifiques roles and requirements for detection engineers?</t>
+          <t>Y a-t-il des rôles spécifiques roles and requirements for detection engineers?
+Maturity guidance:
+1 - No specific roles and requirements
+2 - Requirements identified, not formalised in roles
+3 - Requirements identified, role defined but not documented
+4 - Requirements identified, role defined and documented
+5 - Roles formally documented, approved and regularly revised</t>
         </is>
       </c>
     </row>
@@ -10831,7 +11577,13 @@
       <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)ctive cooperation between the les analystes SOC and the detection engineers?</t>
+          <t>Y a-t-il un(e)ctive cooperation between the les analystes SOC and the detection engineers?
+Maturity guidance:
+1 - No cooperation between teams
+2 - Cooperation between teams on an ad-hoc basis
+3 - SOC analysts are informed, no further cooperation
+4 - SOC analysts are informed and review outcomes
+5 - SOC analyst are actively involved in the detection engineering process</t>
         </is>
       </c>
     </row>
@@ -10864,7 +11616,13 @@
       <c r="F356" t="inlineStr"/>
       <c r="G356" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)ctive cooperation between the Threat Intelligence analysts and detection engineers?</t>
+          <t>Y a-t-il un(e)ctive cooperation between the Threat Intelligence analysts and detection engineers?
+Maturity guidance:
+1 - No cooperation between teams
+2 - Cooperation between teams on an ad-hoc basis
+3 - Threat analysts are informed, no further cooperation
+4 - Threat analysts are informed and review outcomes
+5 - Threat analyst are actively involved in the detection engineering process</t>
         </is>
       </c>
     </row>
@@ -10897,7 +11655,13 @@
       <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr">
         <is>
-          <t>Y a-t-il des hand-over to the analyst team?</t>
+          <t>Y a-t-il des hand-over to the analyst team?
+Maturity guidance:
+1 - Formal handover not in place
+2 - Handover performed in an ad-hoc manner
+3 - Handover performed, process not documented of formalised
+4 - Handover performed, process documentation in place
+5 - Formal handover procedure in place, documented and regularly evaluated</t>
         </is>
       </c>
     </row>
@@ -10930,7 +11694,13 @@
       <c r="F358" t="inlineStr"/>
       <c r="G358" t="inlineStr">
         <is>
-          <t>Y a-t-il une procédure de test enviroment to test and validate detections before deploying them?</t>
+          <t>Y a-t-il une procédure de test enviroment to test and validate detections before deploying them?
+Maturity guidance:
+1 - Testing environment not in place
+2 - Testing environment in place, not actively used for detection engineering
+3 - Testing environment used, testing process not documented or formalised
+4 - Testing environment used, testing process documented
+5 - Testing environment used, process documented and regularly evaluated</t>
         </is>
       </c>
     </row>
@@ -10963,7 +11733,13 @@
       <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr">
         <is>
-          <t>Y a-t-il un processus de release formel process en place for new detections?</t>
+          <t>Y a-t-il un processus de release formel process en place for new detections?
+Maturity guidance:
+1 - Release process not in place
+2 - Releases performed in an ad-hoc manner
+3 - Releases done structurally, process not documented of formalised
+4 - Releases done structurally, process documentation in place
+5 - Formal release procedure in place, documented and regularly evaluated</t>
         </is>
       </c>
     </row>
@@ -10996,7 +11772,13 @@
       <c r="F360" t="inlineStr"/>
       <c r="G360" t="inlineStr">
         <is>
-          <t>Appliquez-vous un système de versionnage to detections?</t>
+          <t>Appliquez-vous un système de versionnage to detections?
+Maturity guidance:
+1 - Versioning system not in place
+2 - Versioning system in place, not actively used
+3 - Versioning system used for some detections
+4 - Versioning system used for all detections, no formal commit procedure
+5 - Versioning system used for all detections, commit procedure formalised</t>
         </is>
       </c>
     </row>
@@ -11029,7 +11811,13 @@
       <c r="F361" t="inlineStr"/>
       <c r="G361" t="inlineStr">
         <is>
-          <t>Avez-vous une procédure de retour arrière procedure en place in case of problems with detections?</t>
+          <t>Avez-vous une procédure de retour arrière procedure en place in case of problems with detections?
+Maturity guidance:
+1 - Roll-back procedure not in place
+2 - Roll-back procedure requirements understood, but not operationalized
+3 - Roll-back capability in place, but not documented
+4 - Roll-back capability in place and documented
+5 - Formal roll-back capability in place, documented and regularly tested</t>
         </is>
       </c>
     </row>
@@ -11043,9 +11831,17 @@
           <t>Process.5.2</t>
         </is>
       </c>
-      <c r="D362" t="inlineStr"/>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>[Process.5.2]</t>
+        </is>
+      </c>
       <c r="E362" t="inlineStr"/>
-      <c r="F362" t="inlineStr"/>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>[Process.5.2]</t>
+        </is>
+      </c>
       <c r="G362" t="inlineStr"/>
     </row>
     <row r="363">
@@ -11077,7 +11873,13 @@
       <c r="F363" t="inlineStr"/>
       <c r="G363" t="inlineStr">
         <is>
-          <t>Effectuez-vous une émulation d'adversaire emulation or automated detection testing? [1]</t>
+          <t>Effectuez-vous une émulation d'adversaire emulation or automated detection testing? [1]
+Maturity guidance:
+1 - Validation activities not performed
+2 - Validation activities performed in an ad-hoc fashion
+3 - Validation activities performed structurally, no documented process
+4 - Validation activities performed structurally following a documented process
+5 - Validation activities fully aligned with TI and continuously improved</t>
         </is>
       </c>
     </row>
@@ -11110,28 +11912,7 @@
       <c r="F364" t="inlineStr"/>
       <c r="G364" t="inlineStr">
         <is>
-          <t>Testez-vous la détection des techniques of les techniques MITRE ATT&amp;CK®?</t>
-        </is>
-      </c>
-    </row>
-    <row r="365">
-      <c r="A365" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="B365" t="n">
-        <v>4</v>
-      </c>
-      <c r="C365" t="inlineStr">
-        <is>
-          <t>Process.5.2.3</t>
-        </is>
-      </c>
-      <c r="D365" t="inlineStr"/>
-      <c r="E365" t="inlineStr">
-        <is>
-          <t>Do you test detection analytics not directly associated with MITRE ATT&amp;CK®?
+          <t>Testez-vous la détection des techniques of les techniques MITRE ATT&amp;CK®?
 Maturity guidance:
 1 - Use case testing not in place
 2 - Use case testing performed in ad-hoc fashion, no detection targets set
@@ -11140,10 +11921,43 @@
 5 - All use cases tested, visibility and detection targets used in improvements</t>
         </is>
       </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="B365" t="n">
+        <v>4</v>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Process.5.2.3</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr"/>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Do you test detection analytics not directly associated with MITRE ATT&amp;CK®?
+Maturity guidance:
+1 - Use case testing not in place
+2 - Use case testing performed in ad-hoc fashion, no detection targets set
+3 - Some use case testing performed, detection targets set, no formal process
+4 - All use cases tested, process formalized, detection targets set
+5 - All use cases tested, visibility and detection targets used in improvements</t>
+        </is>
+      </c>
       <c r="F365" t="inlineStr"/>
       <c r="G365" t="inlineStr">
         <is>
-          <t>Testez-vous les analyses de détection analytics not directly associated with MITRE ATT&amp;CK®?</t>
+          <t>Testez-vous les analyses de détection analytics not directly associated with MITRE ATT&amp;CK®?
+Maturity guidance:
+1 - Use case testing not in place
+2 - Use case testing performed in ad-hoc fashion, no detection targets set
+3 - Some use case testing performed, detection targets set, no formal process
+4 - All use cases tested, process formalized, detection targets set
+5 - All use cases tested, visibility and detection targets used in improvements</t>
         </is>
       </c>
     </row>
@@ -11176,7 +11990,13 @@
       <c r="F366" t="inlineStr"/>
       <c r="G366" t="inlineStr">
         <is>
-          <t>Testez-vous les playbooks de réponse playbooks?</t>
+          <t>Testez-vous les playbooks de réponse playbooks?
+Maturity guidance:
+1 - Response playbooks not tested
+2 - Response playbooks tested in an ad-hoc fashion
+3 - Some response playbooks tested, no formal process
+4 - Response playbooks tested structurally following a documented process
+5 - All response playbooks formally tested, output used for improvements</t>
         </is>
       </c>
     </row>
@@ -11209,7 +12029,13 @@
       <c r="F367" t="inlineStr"/>
       <c r="G367" t="inlineStr">
         <is>
-          <t>La validation de détection est-elle validation fully integrated in le processus d'ingénierie de détection / pipeline?</t>
+          <t>La validation de détection est-elle validation fully integrated in le processus d'ingénierie de détection / pipeline?
+Maturity guidance:
+1 - New releases do not trigger ADT/AE
+2 - New releases trigger ADT/AE in an ad-hoc fashion
+3 - Release process triggers ADT/AE for some use cases, not documented
+4 - Releases process triggers ADT/AE for all use cases, documented process
+5 - Full integration into release process, formalized and (partly) automated</t>
         </is>
       </c>
     </row>
@@ -11242,7 +12068,13 @@
       <c r="F368" t="inlineStr"/>
       <c r="G368" t="inlineStr">
         <is>
-          <t>Is the outcome from detection validation utilisé comme entrée dans la surveillance and detection engineering?</t>
+          <t>Is the outcome from detection validation utilisé comme entrée dans la surveillance and detection engineering?
+Maturity guidance:
+1 - ADT/AE outcome not used
+2 - ADT/AE outcome used in an ad-hoc fashion
+3 - ADT/AE outcome used, no documented process
+4 - ADT/AE outcome used, documented process
+5 - ADT/EA outcome used, process documented and regularly evaluated</t>
         </is>
       </c>
     </row>
@@ -11275,7 +12107,13 @@
       <c r="F369" t="inlineStr"/>
       <c r="G369" t="inlineStr">
         <is>
-          <t>Surveillez-vous l'état d'ingestion des données ingestion status for les sources de données?</t>
+          <t>Surveillez-vous l'état d'ingestion des données ingestion status for les sources de données?
+Maturity guidance:
+1 - Data ingestion status not monitored
+2 - Data ingestion status monitored in an ad-hoc fashion
+3 - Data ingestion status monitored, not complete for all data source types
+4 - Data ingestion status monitored for all log sources, failures result in alerts
+5 - Data ingestion status monitored, following a defined resolution process</t>
         </is>
       </c>
     </row>
@@ -11308,7 +12146,13 @@
       <c r="F370" t="inlineStr"/>
       <c r="G370" t="inlineStr">
         <is>
-          <t>Mesurez-vous et gérez-vous activement and improve la couverture des sources de données?</t>
+          <t>Mesurez-vous et gérez-vous activement and improve la couverture des sources de données?
+Maturity guidance:
+1 - Data source coverage not measured
+2 - Data source coverage measured in an ad-hoc fashion
+3 - Data source coverage measured , not complete for all data source types
+4 - Data source coverage structurally measured and improved on
+5 - Data source coverage structurally improved on following a defined process</t>
         </is>
       </c>
     </row>
@@ -11345,9 +12189,17 @@
           <t>Process.6.1</t>
         </is>
       </c>
-      <c r="D372" t="inlineStr"/>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>[Process.6.1]</t>
+        </is>
+      </c>
       <c r="E372" t="inlineStr"/>
-      <c r="F372" t="inlineStr"/>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>[Process.6.1]</t>
+        </is>
+      </c>
       <c r="G372" t="inlineStr"/>
     </row>
     <row r="373">
@@ -11379,7 +12231,13 @@
       <c r="F373" t="inlineStr"/>
       <c r="G373" t="inlineStr">
         <is>
-          <t>Avez-vous un(e)n automation engineering process en place?</t>
+          <t>Avez-vous un(e)n automation engineering process en place?
+Maturity guidance:
+1 - An automation engineering process is not in place
+2 - Automation engineering is done in an ad-hoc fashion
+3 - Basic process in place, not applied to all task areas
+4 - Informal process in place covering all task areas
+5 - Formal process in place, covering all task areas</t>
         </is>
       </c>
     </row>
@@ -11412,7 +12270,13 @@
       <c r="F374" t="inlineStr"/>
       <c r="G374" t="inlineStr">
         <is>
-          <t>L'automatisation est-elle engineering process formellement documenté?</t>
+          <t>L'automatisation est-elle engineering process formellement documenté?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of automation engineering process
+4 - Single document, full description of automation engineering process
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -11684,7 +12548,13 @@
       <c r="F384" t="inlineStr"/>
       <c r="G384" t="inlineStr">
         <is>
-          <t>Y a-t-il des rôles spécifiques roles and requirements for automation engineers?</t>
+          <t>Y a-t-il des rôles spécifiques roles and requirements for automation engineers?
+Maturity guidance:
+1 - No specific roles and requirements
+2 - Requirements identified, not formalised in roles
+3 - Requirements identified, role defined but not documented
+4 - Requirements identified, role defined and documented
+5 - Roles formally documented, approved and regularly revised</t>
         </is>
       </c>
     </row>
@@ -11717,7 +12587,13 @@
       <c r="F385" t="inlineStr"/>
       <c r="G385" t="inlineStr">
         <is>
-          <t>Les automatisations sont-elles tracked and measured using defined metrics?</t>
+          <t>Les automatisations sont-elles tracked and measured using defined metrics?
+Maturity guidance:
+1 - No metrics in place
+2 - Some measurements performed on ad-hoc basis
+3 - Metrics defined, measurements not consistently performed
+4 - Measurements continuously performed, follow-up not consistent
+5 - Continuous measurement, connected to continuous improvement</t>
         </is>
       </c>
     </row>
@@ -11750,7 +12626,13 @@
       <c r="F386" t="inlineStr"/>
       <c r="G386" t="inlineStr">
         <is>
-          <t>Tous les cas d'usage du SOC sont-ils use cases touched or resolved par automatisation?</t>
+          <t>Tous les cas d'usage du SOC sont-ils use cases touched or resolved par automatisation?
+Maturity guidance:
+1 - No automation applied to SOC use cases
+2 - Automation applied only to selected use cases
+3 - Most SOC use cases applied by generic automation (i.e. enrichment only)
+4 - Most SOC use cases (80%) touched or resolved by specific automation
+5 - All SOC use cases (+95%) touched or resolved by specific automation</t>
         </is>
       </c>
     </row>
@@ -11783,7 +12665,13 @@
       <c r="F387" t="inlineStr"/>
       <c r="G387" t="inlineStr">
         <is>
-          <t>Des playbooks d'automatisation personnalisés automation playbooks développés dans le SOC?</t>
+          <t>Des playbooks d'automatisation personnalisés automation playbooks développés dans le SOC?
+Maturity guidance:
+1 - No custom automation development
+2 - Customization of out-of-the-box automation playbooks
+3 - Playbook development in place, limited application
+4 - Playbooks development process formalised and consistently performed
+5 - Full playbook development process, measured and improved</t>
         </is>
       </c>
     </row>
@@ -11816,7 +12704,13 @@
       <c r="F388" t="inlineStr"/>
       <c r="G388" t="inlineStr">
         <is>
-          <t>Y a-t-il une procédure de test procedure to test and validate automations?</t>
+          <t>Y a-t-il une procédure de test procedure to test and validate automations?
+Maturity guidance:
+1 - No testing performed
+2 - Testing performed in an ad-hoc manner
+3 - Testing procedure defined, not applied consistently
+4 - Testing procedure fully operational, applied consistently
+5 - Testing procedure fully operational, documented and regularly evaluated</t>
         </is>
       </c>
     </row>
@@ -11849,7 +12743,13 @@
       <c r="F389" t="inlineStr"/>
       <c r="G389" t="inlineStr">
         <is>
-          <t>Y a-t-il un processus de release formel process en place for new automations?</t>
+          <t>Y a-t-il un processus de release formel process en place for new automations?
+Maturity guidance:
+1 - Release process not in place
+2 - Releases performed in an ad-hoc manner
+3 - Releases done structurally, process not documented of formalised
+4 - Releases done structurally, process documentation in place
+5 - Formal release procedure in place, documented and regularly evaluated</t>
         </is>
       </c>
     </row>
@@ -11863,9 +12763,17 @@
           <t>Process.6.2</t>
         </is>
       </c>
-      <c r="D390" t="inlineStr"/>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>[Process.6.2]</t>
+        </is>
+      </c>
       <c r="E390" t="inlineStr"/>
-      <c r="F390" t="inlineStr"/>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>[Process.6.2]</t>
+        </is>
+      </c>
       <c r="G390" t="inlineStr"/>
     </row>
     <row r="391">
@@ -11897,7 +12805,13 @@
       <c r="F391" t="inlineStr"/>
       <c r="G391" t="inlineStr">
         <is>
-          <t>Avez-vous une stratégie IA adoption strategy pour le SOC en place?</t>
+          <t>Avez-vous une stratégie IA adoption strategy pour le SOC en place?
+Maturity guidance:
+1 - No AI adoption strategy in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of AI adoption strategy
+4 - Single document, full description of AI adoption strategy
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -12142,7 +13056,13 @@
       <c r="F400" t="inlineStr"/>
       <c r="G400" t="inlineStr">
         <is>
-          <t>La stratégie IA est-elle adoption strategy alignée en interne et approuvée par les parties prenantes?</t>
+          <t>La stratégie IA est-elle adoption strategy alignée en interne et approuvée par les parties prenantes?
+Maturity guidance:
+1 - No internal alignment or approval
+2 - Initial ad-hoc conversations with internal stakeholders completed
+3 - Some alignment in place, not complete or approved
+4 - SOC AI strategy aligned with stakeholders, not formally approved
+5 - SOC AI strategy fully aligned with broader AI strategy, formally approved</t>
         </is>
       </c>
     </row>
@@ -12198,7 +13118,13 @@
       <c r="F402" t="inlineStr"/>
       <c r="G402" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e) log management process en place?</t>
+          <t>Y a-t-il un(e) log management process en place?
+Maturity guidance:
+1 - Log management process is not in place
+2 - Log management is done in an ad-hoc fashion
+3 - Log management process in place, but not applied structurally
+4 - Log management process in place addressing most requirements
+5 - Log management process in place, all requirements met, formally approved</t>
         </is>
       </c>
     </row>
@@ -12231,7 +13157,13 @@
       <c r="F403" t="inlineStr"/>
       <c r="G403" t="inlineStr">
         <is>
-          <t>Are log management elements formellement identifiés et documentés?</t>
+          <t>Are log management elements formellement identifiés et documentés?
+Maturity guidance:
+1 - No log management elements identified
+2 - Some elements identified, managed in ad-hoc fashion
+3 - Most elements identified, no structured approach
+4 - Most elements identified, no managed with a structured approach
+5 - All elements identified, and actively managed through a defined process</t>
         </is>
       </c>
     </row>
@@ -12557,7 +13489,13 @@
       <c r="F415" t="inlineStr"/>
       <c r="G415" t="inlineStr">
         <is>
-          <t>Is the log management process supported by corporate policy?</t>
+          <t>Is the log management process supported by corporate policy?
+Maturity guidance:
+1 - No policy is in place
+2 - Log management requirements scattered across documents
+3 - A policy exists, but has not been accepted formally
+4 - A formal policy exists, but is not actively enforced
+5 - A formal policy exists, actively enforced and supported by stakeholders</t>
         </is>
       </c>
     </row>
@@ -12590,7 +13528,13 @@
       <c r="F416" t="inlineStr"/>
       <c r="G416" t="inlineStr">
         <is>
-          <t>Is the log management process supported by appropriate centralised log management tooling?</t>
+          <t>Is the log management process supported by appropriate centralised log management tooling?
+Maturity guidance:
+1 - No tooling in place
+2 - Log management implemented using a variety of tools
+3 - Centralized tooling in place, configured for basic log management
+4 - Centralized tooling in place, managed and meeting most requirements
+5 - Centralized tooling in place, managed, and optimized for log management</t>
         </is>
       </c>
     </row>
@@ -12623,7 +13567,13 @@
       <c r="F417" t="inlineStr"/>
       <c r="G417" t="inlineStr">
         <is>
-          <t>Is the log management process compliant with applicable standards &amp; regulations?</t>
+          <t>Is the log management process compliant with applicable standards &amp; regulations?
+Maturity guidance:
+1 - Regulations are not known and the process is non-compliant
+2 - Some regulations are known and the process is non-compliant
+3 - Most regulations are known and the process is partially compliant
+4 - Regulations are fully known and the process is mostly compliant
+5 - Regulations are fully known and the process is fully compliant</t>
         </is>
       </c>
     </row>
@@ -12656,7 +13606,13 @@
       <c r="F418" t="inlineStr"/>
       <c r="G418" t="inlineStr">
         <is>
-          <t>Is the log management process aligné avec toutes les parties prenantes?</t>
+          <t>Is the log management process aligné avec toutes les parties prenantes?
+Maturity guidance:
+1 - Stakeholders are unfamiliar with the process
+2 - Some stakeholders are aware of the process, but not its details
+3 - Process awareness in most stakeholders, but no process alignment
+4 - Process aligned with all relevant stakeholders, no formal approval
+5 - Process aligned with all relevant stakeholders, formal approval in place</t>
         </is>
       </c>
     </row>
@@ -12689,7 +13645,13 @@
       <c r="F419" t="inlineStr"/>
       <c r="G419" t="inlineStr">
         <is>
-          <t>Is logging encrypted in transfer, in use, and at rest?</t>
+          <t>Is logging encrypted in transfer, in use, and at rest?
+Maturity guidance:
+1 - No encryption performed
+2 - Some logging encrypted at rest or in transfer
+3 - Most logging encrypted at rest and in transfer
+4 - All logging encrypted (rest &amp; transfer), encryption keys not formally managed
+5 - All logging encrypted (rest &amp; transfer), encryption keys centrally managed</t>
         </is>
       </c>
     </row>
@@ -12722,7 +13684,13 @@
       <c r="F420" t="inlineStr"/>
       <c r="G420" t="inlineStr">
         <is>
-          <t>L'accès to logging restricted to authorized personnel?</t>
+          <t>L'accès to logging restricted to authorized personnel?
+Maturity guidance:
+1 - Access to the system not restricted
+2 - Basic access control in place
+3 - Granular access rights implemented, not monitored
+4 - Granular access rights implemented and monitored, not reviewed
+5 - Granular access rights implemented, monitored and reviewed regularly</t>
         </is>
       </c>
     </row>
@@ -12742,7 +13710,11 @@
         </is>
       </c>
       <c r="E421" t="inlineStr"/>
-      <c r="F421" t="inlineStr"/>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
       <c r="G421" t="inlineStr"/>
     </row>
     <row r="422">
@@ -19884,7 +20856,11 @@
         </is>
       </c>
       <c r="E687" t="inlineStr"/>
-      <c r="F687" t="inlineStr"/>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
       <c r="G687" t="inlineStr"/>
     </row>
     <row r="688">
@@ -19939,7 +20915,13 @@
       <c r="F689" t="inlineStr"/>
       <c r="G689" t="inlineStr">
         <is>
-          <t>Avez-vous formellement described le service de surveillance de sécurité?</t>
+          <t>Avez-vous formellement described le service de surveillance de sécurité?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of service in place
+4 - Single document, full description of service
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -20292,7 +21274,13 @@
       <c r="F702" t="inlineStr"/>
       <c r="G702" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la qualité?</t>
+          <t>Le service est-il mesuré pour la qualité?
+Maturity guidance:
+1 - Service not measured for quality
+2 - Metrics defined, applied in an ad-hoc fashion
+3 - Metrics defined, applied in a structured but informal fashion
+4 - Metrics formalized and used in regular reports
+5 - Formal and approved metrics in place, feedback used for improvement</t>
         </is>
       </c>
     </row>
@@ -20325,7 +21313,13 @@
       <c r="F703" t="inlineStr"/>
       <c r="G703" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?</t>
+          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?
+Maturity guidance:
+1 - Service not measured
+2 - SLA defined, measured in an ad-hoc fashion
+3 - SLA defined, measured periodically but not reported
+4 - SLA compliance reported periodically, not discussed with customers
+5 - SLA compliance discussed with customers regularly for improvement</t>
         </is>
       </c>
     </row>
@@ -20358,7 +21352,13 @@
       <c r="F704" t="inlineStr"/>
       <c r="G704" t="inlineStr">
         <is>
-          <t>Les clients and/or parties prenantes regularly updated about the service?</t>
+          <t>Les clients and/or parties prenantes regularly updated about the service?
+Maturity guidance:
+1 - No updates sent to customers/stakeholders
+2 - Ad-hoc updates sent to some customers/stakeholders
+3 - Frequent updates sent to most customers/stakeholders
+4 - Periodical updates sent to all customers/stakeholders
+5 - Periodical updates sent and discussed with all customers/stakeholders</t>
         </is>
       </c>
     </row>
@@ -20391,7 +21391,13 @@
       <c r="F705" t="inlineStr"/>
       <c r="G705" t="inlineStr">
         <is>
-          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?</t>
+          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?
+Maturity guidance:
+1 - Contractual agreements not in place
+2 - No contract in place, ad-hoc agreements made
+3 - Basic contract in place, not formally signed of
+4 - Contract signed, but not regularly reviewed
+5 - Contract signed, approved by- and regularly reviewed with customers</t>
         </is>
       </c>
     </row>
@@ -20424,7 +21430,13 @@
       <c r="F706" t="inlineStr"/>
       <c r="G706" t="inlineStr">
         <is>
-          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?</t>
+          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?
+Maturity guidance:
+1 - No personnel allocated
+2 - Personnel allocated, but not sufficient for required service delivery
+3 - Personnel allocated, not dedicated for this service
+4 - Sufficient dedicated personnel available, not fully trained and capable
+5 - Sufficient dedicated personnel available, trained and fully capable</t>
         </is>
       </c>
     </row>
@@ -20457,7 +21469,13 @@
       <c r="F707" t="inlineStr"/>
       <c r="G707" t="inlineStr">
         <is>
-          <t>Le service est-il aligné avec les autres processus pertinents?</t>
+          <t>Le service est-il aligné avec les autres processus pertinents?
+Maturity guidance:
+1 - Process not aligned
+2 - Alignment done in an ad-hoc fashion
+3 - Alignment done regularly, but not in a structured fashion
+4 - Alignment done structurally &amp; regularly with most relevant processes
+5 - Alignment done structurally &amp; regularly with all relevant processes</t>
         </is>
       </c>
     </row>
@@ -20490,7 +21508,13 @@
       <c r="F708" t="inlineStr"/>
       <c r="G708" t="inlineStr">
         <is>
-          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?</t>
+          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?
+Maturity guidance:
+1 - No such process in place
+2 - Continuity requirements identified, process not yet in place
+3 - Basic service continuity process in place
+4 - Full process in place, not approved by relevant stakeholders
+5 - Full process in place, formally approved by relevant stakeholders</t>
         </is>
       </c>
     </row>
@@ -20523,7 +21547,13 @@
       <c r="F709" t="inlineStr"/>
       <c r="G709" t="inlineStr">
         <is>
-          <t>Un ensemble de procédures a-t-il été créé been created for this service?</t>
+          <t>Un ensemble de procédures a-t-il été créé been created for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - All procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and regularly reviewed</t>
         </is>
       </c>
     </row>
@@ -20556,7 +21586,13 @@
       <c r="F710" t="inlineStr"/>
       <c r="G710" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?</t>
+          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - Full procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and regularly reviewed</t>
         </is>
       </c>
     </row>
@@ -20589,7 +21625,13 @@
       <c r="F711" t="inlineStr"/>
       <c r="G711" t="inlineStr">
         <is>
-          <t>Les meilleures pratiques sont-elles applied to the service?</t>
+          <t>Les meilleures pratiques sont-elles applied to the service?
+Maturity guidance:
+1 - Best practices not applied
+2 - Best practices identified, but not applied
+3 - Best practices applied, but not structurally
+4 - Best practices applied to service architecture and service delivery
+5 - Best practices applied and adherence checked regularly</t>
         </is>
       </c>
     </row>
@@ -20622,7 +21664,13 @@
       <c r="F712" t="inlineStr"/>
       <c r="G712" t="inlineStr">
         <is>
-          <t>Les cas d'usage sont-ils used in le service de surveillance de sécurité?</t>
+          <t>Les cas d'usage sont-ils used in le service de surveillance de sécurité?
+Maturity guidance:
+1 - Use cases not used
+2 - Use cases undocumented and used in an ad-hoc fashion
+3 - Use cases documented and applied structurally
+4 - Use cases embedded in the security monitoring processes
+5 - Use cases fully embedded, tuning and Life Cycle Management applied</t>
         </is>
       </c>
     </row>
@@ -20655,7 +21703,13 @@
       <c r="F713" t="inlineStr"/>
       <c r="G713" t="inlineStr">
         <is>
-          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?</t>
+          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?
+Maturity guidance:
+1 - Service performance not measured
+2 - Goals set for service performance, measured ad-hoc
+3 - Goals set for service performance, measured structurally but informally
+4 - Goals set for service performance, measured structurally and formally
+5 - Continuous measurement to determine progress &amp; adjust process</t>
         </is>
       </c>
     </row>
@@ -20688,7 +21742,13 @@
       <c r="F714" t="inlineStr"/>
       <c r="G714" t="inlineStr">
         <is>
-          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?</t>
+          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?
+Maturity guidance:
+1 - Improvement not done
+2 - Goals defined, but not pursued
+3 - Goals defined and pursued structurally, but not formalized
+4 - Goals formally defined and pursued structurally and periodically
+5 - Continuous improvement based on targets and feedback loops</t>
         </is>
       </c>
     </row>
@@ -21569,7 +22629,13 @@
       <c r="F747" t="inlineStr"/>
       <c r="G747" t="inlineStr">
         <is>
-          <t>Avez-vous adopted a standard for the Security Incident Management process?</t>
+          <t>Avez-vous adopted a standard for the Security Incident Management process?
+Maturity guidance:
+1 - Standard not adopted
+2 - Awareness of standards, used in ad-hoc fashion
+3 - Standard used structurally as reference during incident response
+4 - Many elements adopted, not fully aligned
+5 - Standard fully adopted, process set up and executed using standard</t>
         </is>
       </c>
     </row>
@@ -21602,7 +22668,13 @@
       <c r="F748" t="inlineStr"/>
       <c r="G748" t="inlineStr">
         <is>
-          <t>Avez-vous formellement described l'incident de sécurité management process?</t>
+          <t>Avez-vous formellement described l'incident de sécurité management process?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of service in place
+4 - Single document, full description of service
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -21955,7 +23027,13 @@
       <c r="F761" t="inlineStr"/>
       <c r="G761" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la qualité?</t>
+          <t>Le service est-il mesuré pour la qualité?
+Maturity guidance:
+1 - Service not measured for quality
+2 - Metrics defined, applied in an ad-hoc fashion
+3 - Metrics defined, applied in a structured but informal fashion
+4 - Metrics formalized and used in regular reports
+5 - Formal and approved metrics in place, feedback used for improvement</t>
         </is>
       </c>
     </row>
@@ -21988,7 +23066,13 @@
       <c r="F762" t="inlineStr"/>
       <c r="G762" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?</t>
+          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?
+Maturity guidance:
+1 - Service not measured
+2 - SLA defined, measured in an ad-hoc fashion
+3 - SLA defined, measured periodically but not reported
+4 - SLA compliance reported periodically, not discussed with customers
+5 - SLA compliance discussed with customers regularly for improvement</t>
         </is>
       </c>
     </row>
@@ -22021,7 +23105,13 @@
       <c r="F763" t="inlineStr"/>
       <c r="G763" t="inlineStr">
         <is>
-          <t>Les clients and/or parties prenantes regularly updated about the service?</t>
+          <t>Les clients and/or parties prenantes regularly updated about the service?
+Maturity guidance:
+1 - No updates sent to customers/stakeholders
+2 - Ad-hoc updates sent to some customers/stakeholders
+3 - Frequent updates sent to most customers/stakeholders
+4 - Periodical updates sent to all customers/stakeholders
+5 - Periodical updates sent and discussed with all customers/stakeholders</t>
         </is>
       </c>
     </row>
@@ -22054,7 +23144,13 @@
       <c r="F764" t="inlineStr"/>
       <c r="G764" t="inlineStr">
         <is>
-          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?</t>
+          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?
+Maturity guidance:
+1 - Contractual agreements not in place
+2 - No contract in place, ad-hoc agreements made
+3 - Basic contract in place, not formally signed of
+4 - Contract signed, but not regularly reviewed
+5 - Contract signed, approved by- and regularly reviewed with customers</t>
         </is>
       </c>
     </row>
@@ -22087,7 +23183,13 @@
       <c r="F765" t="inlineStr"/>
       <c r="G765" t="inlineStr">
         <is>
-          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?</t>
+          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?
+Maturity guidance:
+1 - No personnel allocated
+2 - Personnel allocated, but not sufficient for required service delivery
+3 - Personnel allocated, not dedicated for this service
+4 - Sufficient dedicated personnel available, not fully trained and capable
+5 - Sufficient dedicated personnel available, trained and fully capable</t>
         </is>
       </c>
     </row>
@@ -22120,7 +23222,13 @@
       <c r="F766" t="inlineStr"/>
       <c r="G766" t="inlineStr">
         <is>
-          <t>Le service est-il aligné avec les autres processus pertinents?</t>
+          <t>Le service est-il aligné avec les autres processus pertinents?
+Maturity guidance:
+1 - Process not aligned
+2 - Alignment done in an ad-hoc fashion
+3 - Alignment done regularly, but not in a structured fashion
+4 - Alignment done structurally &amp; regularly with most relevant processes
+5 - Alignment done structurally &amp; regularly with all relevant processes</t>
         </is>
       </c>
     </row>
@@ -22153,7 +23261,13 @@
       <c r="F767" t="inlineStr"/>
       <c r="G767" t="inlineStr">
         <is>
-          <t>Le processus d'incident est-il response team authorized to perform (invasive) actions when required?</t>
+          <t>Le processus d'incident est-il response team authorized to perform (invasive) actions when required?
+Maturity guidance:
+1 - No mandate
+2 - Mandate requested in ad-hoc fashion during incident response
+3 - Mandate informally given, not supported by all stakeholders
+4 - Mandate given and supported by all stakeholders, not formalized
+5 - Full mandate, formally documented, approved and published</t>
         </is>
       </c>
     </row>
@@ -22186,7 +23300,13 @@
       <c r="F768" t="inlineStr"/>
       <c r="G768" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?</t>
+          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - Full procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and regularly reviewed</t>
         </is>
       </c>
     </row>
@@ -22219,7 +23339,13 @@
       <c r="F769" t="inlineStr"/>
       <c r="G769" t="inlineStr">
         <is>
-          <t>Les meilleures pratiques sont-elles applied to the service?</t>
+          <t>Les meilleures pratiques sont-elles applied to the service?
+Maturity guidance:
+1 - Best practices not applied
+2 - Best practices identified, but not applied
+3 - Best practices applied, but not structurally
+4 - Best practices applied to service architecture and service delivery
+5 - Best practices applied and adherence checked regularly</t>
         </is>
       </c>
     </row>
@@ -22252,7 +23378,13 @@
       <c r="F770" t="inlineStr"/>
       <c r="G770" t="inlineStr">
         <is>
-          <t>Le service est-il supported by predefined workflows or scenarios?</t>
+          <t>Le service est-il supported by predefined workflows or scenarios?
+Maturity guidance:
+1 - No workflows or scenarios in place
+2 - Some ad-hoc information across documents
+3 - Basic workflows in place, not covering all incident types
+4 - Workflows created for all incident types, not formalized
+5 - Formal workflows created, approved &amp; published for all incident types</t>
         </is>
       </c>
     </row>
@@ -22285,7 +23417,13 @@
       <c r="F771" t="inlineStr"/>
       <c r="G771" t="inlineStr">
         <is>
-          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?</t>
+          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?
+Maturity guidance:
+1 - Service performance not measured
+2 - Goals set for service performance, measured ad-hoc
+3 - Goals set for service performance, measured structurally but informally
+4 - Goals set for service performance, measured structurally and formally
+5 - Continuous measurement to determine progress &amp; adjust process</t>
         </is>
       </c>
     </row>
@@ -22318,7 +23456,13 @@
       <c r="F772" t="inlineStr"/>
       <c r="G772" t="inlineStr">
         <is>
-          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?</t>
+          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?
+Maturity guidance:
+1 - Improvement not done
+2 - Goals defined, but not pursued
+3 - Goals defined and pursued structurally, but not formalized
+4 - Goals formally defined and pursued structurally and periodically
+5 - Continuous improvement based on targets and feedback loops</t>
         </is>
       </c>
     </row>
@@ -23369,7 +24513,13 @@
       <c r="F811" t="inlineStr"/>
       <c r="G811" t="inlineStr">
         <is>
-          <t>Avez-vous formellement described the forensic analysis service?</t>
+          <t>Avez-vous formellement described the forensic analysis service?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of service in place
+4 - Single document, full description of service
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -23722,7 +24872,13 @@
       <c r="F824" t="inlineStr"/>
       <c r="G824" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la qualité?</t>
+          <t>Le service est-il mesuré pour la qualité?
+Maturity guidance:
+1 - Service not measured for quality
+2 - Metrics defined, applied in an ad-hoc fashion
+3 - Metrics defined, applied in a structured but informal fashion
+4 - Metrics formalized and used in regular reports
+5 - Formal and approved metrics in place, feedback used for improvement</t>
         </is>
       </c>
     </row>
@@ -23755,7 +24911,13 @@
       <c r="F825" t="inlineStr"/>
       <c r="G825" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?</t>
+          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?
+Maturity guidance:
+1 - Service not measured
+2 - SLA defined, measured in an ad-hoc fashion
+3 - SLA defined, measured periodically but not reported
+4 - SLA compliance reported periodically, not discussed with customers
+5 - SLA compliance discussed with customers regularly for improvement</t>
         </is>
       </c>
     </row>
@@ -23788,7 +24950,13 @@
       <c r="F826" t="inlineStr"/>
       <c r="G826" t="inlineStr">
         <is>
-          <t>Les clients and/or parties prenantes regularly updated about the service?</t>
+          <t>Les clients and/or parties prenantes regularly updated about the service?
+Maturity guidance:
+1 - No updates sent to customers/stakeholders
+2 - Ad-hoc updates sent to some customers/stakeholders
+3 - Frequent updates sent to most customers/stakeholders
+4 - Periodical updates sent to all customers/stakeholders
+5 - Periodical updates sent and discussed with all customers/stakeholders</t>
         </is>
       </c>
     </row>
@@ -23821,7 +24989,13 @@
       <c r="F827" t="inlineStr"/>
       <c r="G827" t="inlineStr">
         <is>
-          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?</t>
+          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?
+Maturity guidance:
+1 - Contractual agreements not in place
+2 - No contract in place, ad-hoc agreements made
+3 - Basic contract in place, not formally signed of
+4 - Contract signed, but not regularly reviewed
+5 - Contract signed, approved by- and regularly reviewed with customers</t>
         </is>
       </c>
     </row>
@@ -23854,7 +25028,13 @@
       <c r="F828" t="inlineStr"/>
       <c r="G828" t="inlineStr">
         <is>
-          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?</t>
+          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?
+Maturity guidance:
+1 - No personnel allocated
+2 - Personnel allocated, but not sufficient for required service delivery
+3 - Personnel allocated, not dedicated for this service
+4 - Sufficient dedicated personnel available, not fully trained and capable
+5 - Sufficient dedicated personnel available, trained and fully capable</t>
         </is>
       </c>
     </row>
@@ -23887,7 +25067,13 @@
       <c r="F829" t="inlineStr"/>
       <c r="G829" t="inlineStr">
         <is>
-          <t>Le service est-il aligné avec les autres processus pertinents?</t>
+          <t>Le service est-il aligné avec les autres processus pertinents?
+Maturity guidance:
+1 - Process not aligned
+2 - Alignment done in an ad-hoc fashion
+3 - Alignment done regularly, but not in a structured fashion
+4 - Alignment done structurally &amp; regularly with most relevant processes
+5 - Alignment done structurally &amp; regularly with all relevant processes</t>
         </is>
       </c>
     </row>
@@ -23920,7 +25106,13 @@
       <c r="F830" t="inlineStr"/>
       <c r="G830" t="inlineStr">
         <is>
-          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?</t>
+          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?
+Maturity guidance:
+1 - No such process in place
+2 - Continuity requirements identified, process not yet in place
+3 - Basic service continuity process in place
+4 - Full process in place, not approved by relevant stakeholders
+5 - Full process in place, formally approved by relevant stakeholders</t>
         </is>
       </c>
     </row>
@@ -23953,7 +25145,13 @@
       <c r="F831" t="inlineStr"/>
       <c r="G831" t="inlineStr">
         <is>
-          <t>Un ensemble de procédures a-t-il été créé been created for this service?</t>
+          <t>Un ensemble de procédures a-t-il été créé been created for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - All procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and fully operationalized</t>
         </is>
       </c>
     </row>
@@ -23986,7 +25184,13 @@
       <c r="F832" t="inlineStr"/>
       <c r="G832" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?</t>
+          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - Full procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and regularly reviewed</t>
         </is>
       </c>
     </row>
@@ -24019,7 +25223,13 @@
       <c r="F833" t="inlineStr"/>
       <c r="G833" t="inlineStr">
         <is>
-          <t>Les meilleures pratiques sont-elles applied to the service?</t>
+          <t>Les meilleures pratiques sont-elles applied to the service?
+Maturity guidance:
+1 - No workflows or scenarios in place
+2 - Some ad-hoc information across documents
+3 - Basic workflows in place, not covering all incident types
+4 - Workflows created for all incident types, not formalized
+5 - Formal workflows created, approved and published for all incident types</t>
         </is>
       </c>
     </row>
@@ -24052,7 +25262,13 @@
       <c r="F834" t="inlineStr"/>
       <c r="G834" t="inlineStr">
         <is>
-          <t>Le service est-il supported by predefined workflows or scenarios?</t>
+          <t>Le service est-il supported by predefined workflows or scenarios?
+Maturity guidance:
+1 - Service performance not measured
+2 - Goals set for service performance, measured ad-hoc
+3 - Goals set for service performance, measured structurally but informally
+4 - Goals set for service performance, measured structurally and formally
+5 - Continuous measurement to determine progress &amp; adjust process</t>
         </is>
       </c>
     </row>
@@ -24085,7 +25301,13 @@
       <c r="F835" t="inlineStr"/>
       <c r="G835" t="inlineStr">
         <is>
-          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?</t>
+          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?
+Maturity guidance:
+1 - Improvement not done
+2 - Goals defined, but not pursued
+3 - Goals defined and pursued structurally, but not formalized
+4 - Goals formally defined and pursued structurally and periodically
+5 - Continuous improvement based on targets and feedback loops</t>
         </is>
       </c>
     </row>
@@ -24839,7 +26061,13 @@
       <c r="F863" t="inlineStr"/>
       <c r="G863" t="inlineStr">
         <is>
-          <t>Avez-vous formellement described the threat intelligence service?</t>
+          <t>Avez-vous formellement described the threat intelligence service?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of service in place
+4 - Single document, full description of service
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -25192,7 +26420,13 @@
       <c r="F876" t="inlineStr"/>
       <c r="G876" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la qualité?</t>
+          <t>Le service est-il mesuré pour la qualité?
+Maturity guidance:
+1 - Service not measured for quality
+2 - Metrics defined, applied in an ad-hoc fashion
+3 - Metrics defined, applied in a structured but informal fashion
+4 - Metrics formalized and used in regular reports
+5 - Formal and approved metrics in place, feedback used for improvement</t>
         </is>
       </c>
     </row>
@@ -25225,7 +26459,13 @@
       <c r="F877" t="inlineStr"/>
       <c r="G877" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?</t>
+          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?
+Maturity guidance:
+1 - Service not measured
+2 - SLA defined, measured in an ad-hoc fashion
+3 - SLA defined, measured periodically but not reported
+4 - SLA compliance reported periodically, not discussed with customers
+5 - SLA compliance discussed with customers regularly for improvement</t>
         </is>
       </c>
     </row>
@@ -25258,7 +26498,13 @@
       <c r="F878" t="inlineStr"/>
       <c r="G878" t="inlineStr">
         <is>
-          <t>Les clients and/or parties prenantes regularly updated about the service?</t>
+          <t>Les clients and/or parties prenantes regularly updated about the service?
+Maturity guidance:
+1 - No updates sent to customers/stakeholders
+2 - Ad-hoc updates sent to some customers/stakeholders
+3 - Frequent updates sent to most customers/stakeholders
+4 - Periodical updates sent to all customers/stakeholders
+5 - Periodical updates sent and discussed with all customers/stakeholders</t>
         </is>
       </c>
     </row>
@@ -25291,7 +26537,13 @@
       <c r="F879" t="inlineStr"/>
       <c r="G879" t="inlineStr">
         <is>
-          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?</t>
+          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?
+Maturity guidance:
+1 - Contractual agreements not in place
+2 - No contract in place, ad-hoc agreements made
+3 - Basic contract in place, not formally signed of
+4 - Contract signed, but not regularly reviewed
+5 - Contract signed, approved by- and regularly reviewed with customers</t>
         </is>
       </c>
     </row>
@@ -25324,7 +26576,13 @@
       <c r="F880" t="inlineStr"/>
       <c r="G880" t="inlineStr">
         <is>
-          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?</t>
+          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?
+Maturity guidance:
+1 - No personnel allocated
+2 - Personnel allocated, but not sufficient for required service delivery
+3 - Personnel allocated, not dedicated for this service
+4 - Sufficient dedicated personnel available, not fully trained and capable
+5 - Sufficient dedicated personnel available, trained and fully capable</t>
         </is>
       </c>
     </row>
@@ -25357,7 +26615,13 @@
       <c r="F881" t="inlineStr"/>
       <c r="G881" t="inlineStr">
         <is>
-          <t>Le service est-il aligné avec les autres processus pertinents?</t>
+          <t>Le service est-il aligné avec les autres processus pertinents?
+Maturity guidance:
+1 - Process not aligned
+2 - Alignment done in an ad-hoc fashion
+3 - Alignment done regularly, but not in a structured fashion
+4 - Alignment done structurally &amp; regularly with most relevant processes
+5 - Alignment done structurally &amp; regularly with all relevant processes</t>
         </is>
       </c>
     </row>
@@ -25390,7 +26654,13 @@
       <c r="F882" t="inlineStr"/>
       <c r="G882" t="inlineStr">
         <is>
-          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?</t>
+          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?
+Maturity guidance:
+1 - No such process in place
+2 - Continuity requirements identified, process not yet in place
+3 - Basic service continuity process in place
+4 - Full process in place, not approved by relevant stakeholders
+5 - Full process in place, formally approved by relevant stakeholders</t>
         </is>
       </c>
     </row>
@@ -25423,7 +26693,13 @@
       <c r="F883" t="inlineStr"/>
       <c r="G883" t="inlineStr">
         <is>
-          <t>Un ensemble de procédures a-t-il été créé been created for this service?</t>
+          <t>Un ensemble de procédures a-t-il été créé been created for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - All procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and fully operationalized</t>
         </is>
       </c>
     </row>
@@ -25456,7 +26732,13 @@
       <c r="F884" t="inlineStr"/>
       <c r="G884" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?</t>
+          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - Full procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and regularly reviewed</t>
         </is>
       </c>
     </row>
@@ -25489,7 +26771,13 @@
       <c r="F885" t="inlineStr"/>
       <c r="G885" t="inlineStr">
         <is>
-          <t>Les meilleures pratiques sont-elles applied to the service?</t>
+          <t>Les meilleures pratiques sont-elles applied to the service?
+Maturity guidance:
+1 - Best practices not applied
+2 - Best practices identified, but not applied
+3 - Best practices applied, but not structurally
+4 - Best practices applied to service architecture and service delivery
+5 - Best practices applied and adherence checked regularly</t>
         </is>
       </c>
     </row>
@@ -25522,7 +26810,13 @@
       <c r="F886" t="inlineStr"/>
       <c r="G886" t="inlineStr">
         <is>
-          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?</t>
+          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?
+Maturity guidance:
+1 - Service performance not measured
+2 - Goals set for service performance, measured ad-hoc
+3 - Goals set for service performance, measured structurally but informally
+4 - Goals set for service performance, measured structurally and formally
+5 - Continuous measurement to determine progress &amp; adjust process</t>
         </is>
       </c>
     </row>
@@ -25555,7 +26849,13 @@
       <c r="F887" t="inlineStr"/>
       <c r="G887" t="inlineStr">
         <is>
-          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?</t>
+          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?
+Maturity guidance:
+1 - Improvement not done
+2 - Goals defined, but not pursued
+3 - Goals defined and pursued structurally, but not formalized
+4 - Goals formally defined and pursued structurally and periodically
+5 - Continuous improvement based on targets and feedback loops</t>
         </is>
       </c>
     </row>
@@ -26768,7 +28068,13 @@
       <c r="F932" t="inlineStr"/>
       <c r="G932" t="inlineStr">
         <is>
-          <t>Utilisez-vous a standardized threat hunting methodology?</t>
+          <t>Utilisez-vous a standardized threat hunting methodology?
+Maturity guidance:
+1 - Methodology not adopted
+2 - Awareness of methodologies, used in ad-hoc fashion
+3 - Methodologies used structurally as reference during hunting activities
+4 - Many elements adopted, not fully aligned
+5 - Methodology fully adopted, process set up and executed accordingly</t>
         </is>
       </c>
     </row>
@@ -26801,7 +28107,13 @@
       <c r="F933" t="inlineStr"/>
       <c r="G933" t="inlineStr">
         <is>
-          <t>Avez-vous formellement described the threat hunting service?</t>
+          <t>Avez-vous formellement described the threat hunting service?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of service in place
+4 - Single document, full description of service
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -27154,7 +28466,13 @@
       <c r="F946" t="inlineStr"/>
       <c r="G946" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la qualité?</t>
+          <t>Le service est-il mesuré pour la qualité?
+Maturity guidance:
+1 - Service not measured for quality
+2 - Metrics defined, applied in an ad-hoc fashion
+3 - Metrics defined, applied in a structured but informal fashion
+4 - Metrics formalized and used in regular reports
+5 - Formal and approved metrics in place, feedback used for improvement</t>
         </is>
       </c>
     </row>
@@ -27187,7 +28505,13 @@
       <c r="F947" t="inlineStr"/>
       <c r="G947" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?</t>
+          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?
+Maturity guidance:
+1 - Service not measured
+2 - SLA defined, measured in an ad-hoc fashion
+3 - SLA defined, measured periodically but not reported
+4 - SLA compliance reported periodically, not discussed with customers
+5 - SLA compliance discussed with customers regularly for improvement</t>
         </is>
       </c>
     </row>
@@ -27220,7 +28544,13 @@
       <c r="F948" t="inlineStr"/>
       <c r="G948" t="inlineStr">
         <is>
-          <t>Les clients and/or parties prenantes regularly updated about the service?</t>
+          <t>Les clients and/or parties prenantes regularly updated about the service?
+Maturity guidance:
+1 - No updates sent to customers/stakeholders
+2 - Ad-hoc updates sent to some customers/stakeholders
+3 - Frequent updates sent to most customers/stakeholders
+4 - Periodical updates sent to all customers/stakeholders
+5 - Periodical updates sent and discussed with all customers/stakeholders</t>
         </is>
       </c>
     </row>
@@ -27253,7 +28583,13 @@
       <c r="F949" t="inlineStr"/>
       <c r="G949" t="inlineStr">
         <is>
-          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?</t>
+          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?
+Maturity guidance:
+1 - Contractual agreements not in place
+2 - No contract in place, ad-hoc agreements made
+3 - Basic contract in place, not formally signed of
+4 - Contract signed, but not regularly reviewed
+5 - Contract signed, approved by- and regularly reviewed with customers</t>
         </is>
       </c>
     </row>
@@ -27286,7 +28622,13 @@
       <c r="F950" t="inlineStr"/>
       <c r="G950" t="inlineStr">
         <is>
-          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?</t>
+          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?
+Maturity guidance:
+1 - No personnel allocated
+2 - Personnel allocated, but not sufficient for required service delivery
+3 - Personnel allocated, not dedicated for this service
+4 - Sufficient dedicated personnel available, not fully trained and capable
+5 - Sufficient dedicated personnel available, trained and fully capable</t>
         </is>
       </c>
     </row>
@@ -27319,7 +28661,13 @@
       <c r="F951" t="inlineStr"/>
       <c r="G951" t="inlineStr">
         <is>
-          <t>Le service est-il aligné avec les autres processus pertinents?</t>
+          <t>Le service est-il aligné avec les autres processus pertinents?
+Maturity guidance:
+1 - Process not aligned
+2 - Alignment done in an ad-hoc fashion
+3 - Alignment done regularly, but not in a structured fashion
+4 - Alignment done structurally &amp; regularly with most relevant processes
+5 - Alignment done structurally &amp; regularly with all relevant processes</t>
         </is>
       </c>
     </row>
@@ -27352,7 +28700,13 @@
       <c r="F952" t="inlineStr"/>
       <c r="G952" t="inlineStr">
         <is>
-          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?</t>
+          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?
+Maturity guidance:
+1 - No such process in place
+2 - Continuity requirements identified, process not yet in place
+3 - Basic service continuity process in place
+4 - Full process in place, not approved by relevant stakeholders
+5 - Full process in place, formally approved by relevant stakeholders</t>
         </is>
       </c>
     </row>
@@ -27385,7 +28739,13 @@
       <c r="F953" t="inlineStr"/>
       <c r="G953" t="inlineStr">
         <is>
-          <t>Un ensemble de procédures a-t-il été créé been created for this service?</t>
+          <t>Un ensemble de procédures a-t-il été créé been created for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - All procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and fully operationalized</t>
         </is>
       </c>
     </row>
@@ -27418,7 +28778,13 @@
       <c r="F954" t="inlineStr"/>
       <c r="G954" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?</t>
+          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - Full procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and regularly reviewed</t>
         </is>
       </c>
     </row>
@@ -27451,7 +28817,13 @@
       <c r="F955" t="inlineStr"/>
       <c r="G955" t="inlineStr">
         <is>
-          <t>Les meilleures pratiques sont-elles applied to the service?</t>
+          <t>Les meilleures pratiques sont-elles applied to the service?
+Maturity guidance:
+1 - Best practices not applied
+2 - Best practices identified, but not applied
+3 - Best practices applied, but not structurally
+4 - Best practices applied to service architecture and service delivery
+5 - Best practices applied and adherence checked regularly</t>
         </is>
       </c>
     </row>
@@ -27484,7 +28856,13 @@
       <c r="F956" t="inlineStr"/>
       <c r="G956" t="inlineStr">
         <is>
-          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?</t>
+          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?
+Maturity guidance:
+1 - Service performance not measured
+2 - Goals set for service performance, measured ad-hoc
+3 - Goals set for service performance, measured structurally but informally
+4 - Goals set for service performance, measured structurally and formally
+5 - Continuous measurement to determine progress &amp; adjust process</t>
         </is>
       </c>
     </row>
@@ -27517,7 +28895,13 @@
       <c r="F957" t="inlineStr"/>
       <c r="G957" t="inlineStr">
         <is>
-          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?</t>
+          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?
+Maturity guidance:
+1 - Improvement not done
+2 - Goals defined, but not pursued
+3 - Goals defined and pursued structurally, but not formalized
+4 - Goals formally defined and pursued structurally and periodically
+5 - Continuous improvement based on targets and feedback loops</t>
         </is>
       </c>
     </row>
@@ -28163,7 +29547,13 @@
       <c r="F981" t="inlineStr"/>
       <c r="G981" t="inlineStr">
         <is>
-          <t>Avez-vous formellement described the vulnerability management service?</t>
+          <t>Avez-vous formellement described the vulnerability management service?
+Maturity guidance:
+1 - No documentation in place
+2 - Some ad-hoc information across documents
+3 - Basic documentation of service in place
+4 - Single document, full description of service
+5 - Document completed, approved and formally published</t>
         </is>
       </c>
     </row>
@@ -28516,7 +29906,13 @@
       <c r="F994" t="inlineStr"/>
       <c r="G994" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la qualité?</t>
+          <t>Le service est-il mesuré pour la qualité?
+Maturity guidance:
+1 - Service not measured for quality
+2 - Metrics defined, applied in an ad-hoc fashion
+3 - Metrics defined, applied in a structured but informal fashion
+4 - Metrics formalized and used in regular reports
+5 - Formal and approved metrics in place, feedback used for improvement</t>
         </is>
       </c>
     </row>
@@ -28549,7 +29945,13 @@
       <c r="F995" t="inlineStr"/>
       <c r="G995" t="inlineStr">
         <is>
-          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?</t>
+          <t>Le service est-il mesuré pour la prestation de service in accordance with les niveaux de service?
+Maturity guidance:
+1 - Service not measured
+2 - SLA defined, measured in an ad-hoc fashion
+3 - SLA defined, measured periodically but not reported
+4 - SLA compliance reported periodically, not discussed with customers
+5 - SLA compliance discussed with customers regularly for improvement</t>
         </is>
       </c>
     </row>
@@ -28582,7 +29984,13 @@
       <c r="F996" t="inlineStr"/>
       <c r="G996" t="inlineStr">
         <is>
-          <t>Les clients and/or parties prenantes regularly updated about the service?</t>
+          <t>Les clients and/or parties prenantes regularly updated about the service?
+Maturity guidance:
+1 - No updates sent to customers/stakeholders
+2 - Ad-hoc updates sent to some customers/stakeholders
+3 - Frequent updates sent to most customers/stakeholders
+4 - Periodical updates sent to all customers/stakeholders
+5 - Periodical updates sent and discussed with all customers/stakeholders</t>
         </is>
       </c>
     </row>
@@ -28615,7 +30023,13 @@
       <c r="F997" t="inlineStr"/>
       <c r="G997" t="inlineStr">
         <is>
-          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?</t>
+          <t>Y a-t-il un accord contractuel agreement entre le SOC et les clients?
+Maturity guidance:
+1 - Contractual agreements not in place
+2 - No contract in place, ad-hoc agreements made
+3 - Basic contract in place, not formally signed of
+4 - Contract signed, but not regularly reviewed
+5 - Contract signed, approved by- and regularly reviewed with customers</t>
         </is>
       </c>
     </row>
@@ -28648,7 +30062,13 @@
       <c r="F998" t="inlineStr"/>
       <c r="G998" t="inlineStr">
         <is>
-          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?</t>
+          <t>Le personnel est-il suffisant personnel alloué au processus pour assurer la la prestation de service?
+Maturity guidance:
+1 - No personnel allocated
+2 - Personnel allocated, but not sufficient for required service delivery
+3 - Personnel allocated, not dedicated for this service
+4 - Sufficient dedicated personnel available, not fully trained and capable
+5 - Sufficient dedicated personnel available, trained and fully capable</t>
         </is>
       </c>
     </row>
@@ -28681,7 +30101,13 @@
       <c r="F999" t="inlineStr"/>
       <c r="G999" t="inlineStr">
         <is>
-          <t>Le service est-il aligné avec les autres processus pertinents?</t>
+          <t>Le service est-il aligné avec les autres processus pertinents?
+Maturity guidance:
+1 - Process not aligned
+2 - Alignment done in an ad-hoc fashion
+3 - Alignment done regularly, but not in a structured fashion
+4 - Alignment done structurally &amp; regularly with most relevant processes
+5 - Alignment done structurally &amp; regularly with all relevant processes</t>
         </is>
       </c>
     </row>
@@ -28714,7 +30140,13 @@
       <c r="F1000" t="inlineStr"/>
       <c r="G1000" t="inlineStr">
         <is>
-          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?</t>
+          <t>Y a-t-il un processus d'incident resolution / service continuity process en place pour ce service?
+Maturity guidance:
+1 - No such process in place
+2 - Continuity requirements identified, process not yet in place
+3 - Basic service continuity process in place
+4 - Full process in place, not approved by relevant stakeholders
+5 - Full process in place, formally approved by relevant stakeholders</t>
         </is>
       </c>
     </row>
@@ -28747,7 +30179,13 @@
       <c r="F1001" t="inlineStr"/>
       <c r="G1001" t="inlineStr">
         <is>
-          <t>Un ensemble de procédures a-t-il été créé been created for this service?</t>
+          <t>Un ensemble de procédures a-t-il été créé been created for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - All procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and fully operationalized</t>
         </is>
       </c>
     </row>
@@ -28780,7 +30218,13 @@
       <c r="F1002" t="inlineStr"/>
       <c r="G1002" t="inlineStr">
         <is>
-          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?</t>
+          <t>Y a-t-il un(e)n onboarding and offloading procedure for this service?
+Maturity guidance:
+1 - No procedures in place
+2 - Basic procedures in place, used in an ad-hoc fashion
+3 - Full procedures in place, operational but not used structurally
+4 - Procedures in place, operational and used structurally
+5 - Procedures in place, formally published and regularly reviewed</t>
         </is>
       </c>
     </row>
@@ -28813,7 +30257,13 @@
       <c r="F1003" t="inlineStr"/>
       <c r="G1003" t="inlineStr">
         <is>
-          <t>Les meilleures pratiques sont-elles applied to the service?</t>
+          <t>Les meilleures pratiques sont-elles applied to the service?
+Maturity guidance:
+1 - Best practices not applied
+2 - Best practices identified, but not applied
+3 - Best practices applied, but not structurally
+4 - Best practices applied to service architecture and service delivery
+5 - Best practices applied and adherence checked regularly</t>
         </is>
       </c>
     </row>
@@ -28846,7 +30296,13 @@
       <c r="F1004" t="inlineStr"/>
       <c r="G1004" t="inlineStr">
         <is>
-          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?</t>
+          <t>Les données de processus sont-elles data collectées pour la prédiction of service performance?
+Maturity guidance:
+1 - Service performance not measured
+2 - Goals set for service performance, measured ad-hoc
+3 - Goals set for service performance, measured structurally but informally
+4 - Goals set for service performance, measured structurally and formally
+5 - Continuous measurement to determine progress &amp; adjust process</t>
         </is>
       </c>
     </row>
@@ -28879,7 +30335,13 @@
       <c r="F1005" t="inlineStr"/>
       <c r="G1005" t="inlineStr">
         <is>
-          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?</t>
+          <t>Le service est-il continuellement amélioré basé sur les objectifs d'amélioration?
+Maturity guidance:
+1 - Improvement not done
+2 - Goals defined, but not pursued
+3 - Goals defined and pursued structurally, but not formalized
+4 - Goals formally defined and pursued structurally and periodically
+5 - Continuous improvement based on targets and feedback loops</t>
         </is>
       </c>
     </row>

</xml_diff>